<commit_message>
Import filled rankings (1230 confirmed) and unconfirmed contacts; rebuild workbooks with CONFIRMED/NOT_CONFIRMED split
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WLyHMjDC3dbaNBgTG82etS
</commit_message>
<xml_diff>
--- a/research/brics_universities/output/BRICS_universities_ethiopia.xlsx
+++ b/research/brics_universities/output/BRICS_universities_ethiopia.xlsx
@@ -12,8 +12,8 @@
     <sheet name="Эфиопия" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Волна 1'!$A$1:$AJ$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Эфиопия'!$A$1:$AJ$41</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Волна 1'!$A$1:$AK$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Эфиопия'!$A$1:$AK$41</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -652,7 +652,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AJ4"/>
+  <dimension ref="A1:AK4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -676,21 +676,22 @@
     <col width="13" customWidth="1" min="19" max="19"/>
     <col width="13" customWidth="1" min="20" max="20"/>
     <col width="16" customWidth="1" min="21" max="21"/>
-    <col width="10" customWidth="1" min="22" max="22"/>
-    <col width="45" customWidth="1" min="23" max="23"/>
-    <col width="30" customWidth="1" min="24" max="24"/>
+    <col width="16" customWidth="1" min="22" max="22"/>
+    <col width="10" customWidth="1" min="23" max="23"/>
+    <col width="45" customWidth="1" min="24" max="24"/>
     <col width="30" customWidth="1" min="25" max="25"/>
-    <col width="40" customWidth="1" min="26" max="26"/>
-    <col width="45" customWidth="1" min="27" max="27"/>
-    <col width="22" customWidth="1" min="28" max="28"/>
-    <col width="11" customWidth="1" min="29" max="29"/>
-    <col width="9" customWidth="1" min="30" max="30"/>
-    <col width="12" customWidth="1" min="31" max="31"/>
-    <col width="11" customWidth="1" min="32" max="32"/>
-    <col width="55" customWidth="1" min="33" max="33"/>
-    <col width="60" customWidth="1" min="34" max="34"/>
-    <col width="12" customWidth="1" min="35" max="35"/>
-    <col width="24" customWidth="1" min="36" max="36"/>
+    <col width="30" customWidth="1" min="26" max="26"/>
+    <col width="40" customWidth="1" min="27" max="27"/>
+    <col width="45" customWidth="1" min="28" max="28"/>
+    <col width="22" customWidth="1" min="29" max="29"/>
+    <col width="11" customWidth="1" min="30" max="30"/>
+    <col width="9" customWidth="1" min="31" max="31"/>
+    <col width="12" customWidth="1" min="32" max="32"/>
+    <col width="11" customWidth="1" min="33" max="33"/>
+    <col width="55" customWidth="1" min="34" max="34"/>
+    <col width="60" customWidth="1" min="35" max="35"/>
+    <col width="12" customWidth="1" min="36" max="36"/>
+    <col width="24" customWidth="1" min="37" max="37"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -801,75 +802,80 @@
       </c>
       <c r="V1" s="3" t="inlineStr">
         <is>
+          <t>Рейтинг Webometrics (мир)</t>
+        </is>
+      </c>
+      <c r="W1" s="3" t="inlineStr">
+        <is>
           <t>Запущено КА (спутников)</t>
         </is>
       </c>
-      <c r="W1" s="3" t="inlineStr">
+      <c r="X1" s="3" t="inlineStr">
         <is>
           <t>Названия запущенных КА (год)</t>
         </is>
       </c>
-      <c r="X1" s="3" t="inlineStr">
+      <c r="Y1" s="3" t="inlineStr">
         <is>
           <t>КА в разработке</t>
         </is>
       </c>
-      <c r="Y1" s="3" t="inlineStr">
+      <c r="Z1" s="3" t="inlineStr">
         <is>
           <t>Наземная станция</t>
         </is>
       </c>
-      <c r="Z1" s="3" t="inlineStr">
+      <c r="AA1" s="3" t="inlineStr">
         <is>
           <t>Космические подразделения</t>
         </is>
       </c>
-      <c r="AA1" s="3" t="inlineStr">
+      <c r="AB1" s="3" t="inlineStr">
         <is>
           <t>Партнёрства в космической сфере</t>
         </is>
       </c>
-      <c r="AB1" s="3" t="inlineStr">
+      <c r="AC1" s="3" t="inlineStr">
         <is>
           <t>Санкционные / ограничительные списки (США)</t>
         </is>
       </c>
-      <c r="AC1" s="3" t="inlineStr">
+      <c r="AD1" s="3" t="inlineStr">
         <is>
           <t>Космический индекс (0–100)</t>
         </is>
       </c>
-      <c r="AD1" s="3" t="inlineStr">
+      <c r="AE1" s="3" t="inlineStr">
         <is>
           <t>Волна рассылки</t>
         </is>
       </c>
-      <c r="AE1" s="3" t="inlineStr">
+      <c r="AF1" s="3" t="inlineStr">
         <is>
           <t>Проверка домена e-mail (MX)</t>
         </is>
       </c>
-      <c r="AF1" s="3" t="inlineStr">
+      <c r="AG1" s="3" t="inlineStr">
         <is>
           <t>Достоверность</t>
         </is>
       </c>
-      <c r="AG1" s="3" t="inlineStr">
+      <c r="AH1" s="3" t="inlineStr">
         <is>
           <t>Примечания</t>
         </is>
       </c>
-      <c r="AH1" s="3" t="inlineStr">
+      <c r="AI1" s="3" t="inlineStr">
         <is>
           <t>Источники</t>
         </is>
       </c>
-      <c r="AI1" s="3" t="inlineStr">
+      <c r="AJ1" s="3" t="inlineStr">
         <is>
           <t>Дата проверки</t>
         </is>
       </c>
-      <c r="AJ1" s="3" t="inlineStr">
+      <c r="AK1" s="3" t="inlineStr">
         <is>
           <t>Секретарь парткома (справочно, Китай)</t>
         </is>
@@ -971,31 +977,48 @@
           <t>Director General</t>
         </is>
       </c>
-      <c r="S2" s="4" t="inlineStr"/>
-      <c r="T2" s="4" t="inlineStr"/>
-      <c r="U2" s="4" t="inlineStr"/>
-      <c r="V2" s="4" t="n">
+      <c r="S2" s="4" t="inlineStr">
+        <is>
+          <t>QS2027: не в рейтинге</t>
+        </is>
+      </c>
+      <c r="T2" s="4" t="inlineStr">
+        <is>
+          <t>THE2027: не в рейтинге</t>
+        </is>
+      </c>
+      <c r="U2" s="4" t="inlineStr">
+        <is>
+          <t>нет общенационального рейтинга</t>
+        </is>
+      </c>
+      <c r="V2" s="4" t="inlineStr">
+        <is>
+          <t>нет в опубл. списке</t>
+        </is>
+      </c>
+      <c r="W2" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="W2" s="4" t="inlineStr">
+      <c r="X2" s="4" t="inlineStr">
         <is>
           <t>• ETRSS-1 (2019)
 • ET-SMART-RSS (2020)</t>
         </is>
       </c>
-      <c r="X2" s="4" t="inlineStr">
+      <c r="Y2" s="4" t="inlineStr">
         <is>
           <t>• ETRSS-2 (0.5 m EO satellite, joint development with Shanghai Engineering Center for Microsatellites
 • Launch planned Dec 2026)
 • Domestic satellite AIT centre planned with Roscosmos support</t>
         </is>
       </c>
-      <c r="Y2" s="4" t="inlineStr">
+      <c r="Z2" s="4" t="inlineStr">
         <is>
           <t>Multi-satellite tracking and data-receiving ground station at Entoto (installed May 2021; offered as paid data-reception service); 12-m EO satellite data receiving ground station (built 2024)</t>
         </is>
       </c>
-      <c r="Z2" s="4" t="inlineStr">
+      <c r="AA2" s="4" t="inlineStr">
         <is>
           <t>• Entoto Observatory and Research Center (EORC)
 • Satellite operations/space engineering directorates
@@ -1003,7 +1026,7 @@
 • Postgraduate programs in Astronomy &amp; Astrophysics, Space &amp; Planetary Science, Remote Sensing, Geodesy</t>
         </is>
       </c>
-      <c r="AA2" s="4" t="inlineStr">
+      <c r="AB2" s="4" t="inlineStr">
         <is>
           <t>• Shanghai Engineering Center for Microsatellites (ETRSS-2 contract, Nov 2024)
 • Beijing Smart Satellite Technology (ET-SMART-RSS)
@@ -1013,35 +1036,36 @@
 • FDRE Air Force (agreement)</t>
         </is>
       </c>
-      <c r="AB2" s="4" t="inlineStr"/>
-      <c r="AC2" s="4" t="n">
+      <c r="AC2" s="4" t="inlineStr"/>
+      <c r="AD2" s="4" t="n">
         <v>90</v>
       </c>
-      <c r="AD2" s="5" t="inlineStr">
+      <c r="AE2" s="5" t="inlineStr">
         <is>
           <t>1A</t>
         </is>
       </c>
-      <c r="AE2" s="4" t="inlineStr">
+      <c r="AF2" s="4" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="AF2" s="4" t="inlineStr">
+      <c r="AG2" s="4" t="inlineStr">
         <is>
           <t>высокая</t>
         </is>
       </c>
-      <c r="AG2" s="4" t="inlineStr">
+      <c r="AH2" s="4" t="inlineStr">
         <is>
           <t>• Национальное космическое агентство Эфиопии (бывш. ESSTI + EGII, объединены в 2022); ключевой адресат для созвездия
 • ETRSS-1 (2019) и ET-SMART-RSS (2020) построены в кооперации с Китаем; по данным ENA (янв. 2026) оба завершили срок службы
 • Адрес partnerships@ssgi.gov.et указан на сайте как контакт службы промышленного сотрудничества и партнёрств; отдельного международного отдела на сайте не найдено
 • Написание имени: Abdissa Yilma (сайт SSGI) / Abdisa Yilma (СМИ); на сайте SSGI указан как PhD, Fana пишет 'Mr.'
-• Идут переговоры с Роскосмосом о центре сборки/испытаний спутников (апр. 2026) — благоприятный контекст для БРИКС-сотрудничества</t>
-        </is>
-      </c>
-      <c r="AH2" s="4" t="inlineStr">
+• Идут переговоры с Роскосмосом о центре сборки/испытаний спутников (апр. 2026) — благоприятный контекст для БРИКС-сотрудничества
+• Рейтинги: Национального рейтинга с местами нет: МинОбр Эфиопии делит гос. вузы на категории (research / applied science / general), мест не публикует</t>
+        </is>
+      </c>
+      <c r="AI2" s="4" t="inlineStr">
         <is>
           <t>• Https://ssgi.gov.et
 • Https://ssgi.gov.et/assets/index-CddNteli.js (site leadership/contact data)
@@ -1052,12 +1076,12 @@
 • Nanosats.csv</t>
         </is>
       </c>
-      <c r="AI2" s="4" t="inlineStr">
+      <c r="AJ2" s="4" t="inlineStr">
         <is>
           <t>2026-10-05</t>
         </is>
       </c>
-      <c r="AJ2" s="4" t="inlineStr"/>
+      <c r="AK2" s="4" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
@@ -1156,70 +1180,90 @@
           <t>President</t>
         </is>
       </c>
-      <c r="S3" s="4" t="inlineStr"/>
-      <c r="T3" s="4" t="inlineStr"/>
-      <c r="U3" s="4" t="inlineStr"/>
-      <c r="V3" s="4" t="n">
+      <c r="S3" s="4" t="inlineStr">
+        <is>
+          <t>QS2027: 951–1000</t>
+        </is>
+      </c>
+      <c r="T3" s="4" t="inlineStr">
+        <is>
+          <t>THE2027: не в рейтинге</t>
+        </is>
+      </c>
+      <c r="U3" s="4" t="inlineStr">
+        <is>
+          <t>нет общенационального рейтинга</t>
+        </is>
+      </c>
+      <c r="V3" s="4" t="inlineStr">
+        <is>
+          <t>1109</t>
+        </is>
+      </c>
+      <c r="W3" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="W3" s="4" t="inlineStr"/>
-      <c r="X3" s="4" t="inlineStr">
+      <c r="X3" s="4" t="inlineStr"/>
+      <c r="Y3" s="4" t="inlineStr">
         <is>
           <t>ET-SAT (2U CubeSat by AAiT, pre-selected for QB50) — cancelled, never launched</t>
         </is>
       </c>
-      <c r="Y3" s="4" t="inlineStr"/>
-      <c r="Z3" s="4" t="inlineStr">
+      <c r="Z3" s="4" t="inlineStr"/>
+      <c r="AA3" s="4" t="inlineStr">
         <is>
           <t>• Department of Physics (astrophysics / astronomy research stream)
 • Addis Ababa Institute of Technology — School of Electrical &amp; Computer Engineering (ELEDIA@AAiT research group, communication engineering)</t>
         </is>
       </c>
-      <c r="AA3" s="4" t="inlineStr"/>
       <c r="AB3" s="4" t="inlineStr"/>
-      <c r="AC3" s="4" t="n">
-        <v>25</v>
-      </c>
-      <c r="AD3" s="6" t="inlineStr">
+      <c r="AC3" s="4" t="inlineStr"/>
+      <c r="AD3" s="4" t="n">
+        <v>31</v>
+      </c>
+      <c r="AE3" s="6" t="inlineStr">
         <is>
           <t>1B</t>
         </is>
       </c>
-      <c r="AE3" s="4" t="inlineStr">
+      <c r="AF3" s="4" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="AF3" s="4" t="inlineStr">
+      <c r="AG3" s="4" t="inlineStr">
         <is>
           <t>средняя</t>
         </is>
       </c>
-      <c r="AG3" s="4" t="inlineStr">
+      <c r="AH3" s="4" t="inlineStr">
         <is>
           <t>• Ведущий университет страны; сайт aau.edu.et — JS-приложение, данные взяты из официального API api.aau.edu.et
 • Международными связями ведает Office of Partnerships (подразделение AAU Global) при вице-президенте по партнёрству и коммуникациям; по ENA (фев. 2025) этот пост занимала Dr. Rahel Argaw, в текущем списке руководства на сайте её нет — не подтверждено на 2026
 • Отдельного e-mail президента не опубликовано; email_general — Office of Communication (также в офисе президента, 6 Kilo)
 • QS 2026: 851–900 (fsxbusiness); значение QS 2027 (по поисковой выдаче 951–1000) не подтверждено с открытой страницы — поле оставлено пустым. В THE 2027 по входным данным не ранжирован
-• Спутник ET-SAT (AAiT, QB50) отменён; запусков нет. Почтовый ящик P.O. Box 1176 подтверждён для подразделения AAU (ACEWM), общеуниверситетский P.O. Box стоит перепроверить</t>
-        </is>
-      </c>
-      <c r="AH3" s="4" t="inlineStr">
+• Спутник ET-SAT (AAiT, QB50) отменён; запусков нет. Почтовый ящик P.O. Box 1176 подтверждён для подразделения AAU (ACEWM), общеуниверситетский P.O. Box стоит перепроверить
+• Рейтинги: Национального рейтинга с местами нет: МинОбр Эфиопии делит гос. вузы на категории (research / applied science / general), мест не публикует</t>
+        </is>
+      </c>
+      <c r="AI3" s="4" t="inlineStr">
         <is>
           <t>• Https://api.aau.edu.et/leaderships/
 • Https://api.aau.edu.et/contents/ (Office of Partnerships &amp; Office of Communication pages, updated 2026-04-21)
 • Https://www.ena.et/web/eng/w/eng_6063594
 • Https://www.fsxbusiness.com/aau-tops-east-africa-in-qs-rankings
 • Https://www.nanosats.eu/sat/et-sat
-• Nanosats.csv</t>
-        </is>
-      </c>
-      <c r="AI3" s="4" t="inlineStr">
+• Nanosats.csv
+https://www.topuniversities.com/world-university-rankings (QS WUR 2027)
+https://figshare.com/articles/preprint/Ranking_Web_of_Universities_webometrics_info_July_2026_edition/33062150</t>
+        </is>
+      </c>
+      <c r="AJ3" s="4" t="inlineStr">
         <is>
           <t>2026-10-05</t>
         </is>
       </c>
-      <c r="AJ3" s="4" t="inlineStr"/>
+      <c r="AK3" s="4" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
@@ -1314,73 +1358,92 @@
           <t>President</t>
         </is>
       </c>
-      <c r="S4" s="4" t="inlineStr"/>
-      <c r="T4" s="4" t="inlineStr"/>
-      <c r="U4" s="4" t="inlineStr"/>
-      <c r="V4" s="4" t="n">
+      <c r="S4" s="4" t="inlineStr">
+        <is>
+          <t>QS2027: не в рейтинге</t>
+        </is>
+      </c>
+      <c r="T4" s="4" t="inlineStr">
+        <is>
+          <t>THE2027: не в рейтинге</t>
+        </is>
+      </c>
+      <c r="U4" s="4" t="inlineStr">
+        <is>
+          <t>нет общенационального рейтинга</t>
+        </is>
+      </c>
+      <c r="V4" s="4" t="inlineStr">
+        <is>
+          <t>2237</t>
+        </is>
+      </c>
+      <c r="W4" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="W4" s="4" t="inlineStr"/>
       <c r="X4" s="4" t="inlineStr"/>
-      <c r="Y4" s="4" t="inlineStr">
+      <c r="Y4" s="4" t="inlineStr"/>
+      <c r="Z4" s="4" t="inlineStr">
         <is>
           <t>Blue Nile Radar (BNR) / geospace radar facilities of the Washera Geospace and Radar Science Laboratory</t>
         </is>
       </c>
-      <c r="Z4" s="4" t="inlineStr">
+      <c r="AA4" s="4" t="inlineStr">
         <is>
           <t>• Washera Geospace and Radar Science Laboratory (WaGRL, College of Science)
 • Geospatial Data &amp; Technology Center
 • Bahir Dar Institute of Technology</t>
         </is>
       </c>
-      <c r="AA4" s="4" t="inlineStr"/>
       <c r="AB4" s="4" t="inlineStr"/>
-      <c r="AC4" s="4" t="n">
+      <c r="AC4" s="4" t="inlineStr"/>
+      <c r="AD4" s="4" t="n">
         <v>20</v>
       </c>
-      <c r="AD4" s="6" t="inlineStr">
+      <c r="AE4" s="6" t="inlineStr">
         <is>
           <t>1B</t>
         </is>
       </c>
-      <c r="AE4" s="4" t="inlineStr">
+      <c r="AF4" s="4" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="AF4" s="4" t="inlineStr">
+      <c r="AG4" s="4" t="inlineStr">
         <is>
           <t>средняя</t>
         </is>
       </c>
-      <c r="AG4" s="4" t="inlineStr">
+      <c r="AH4" s="4" t="inlineStr">
         <is>
           <t>• Спутников на орбите не найдено; есть лаборатория геокосмоса и радаров (ионосфера, TEC-модели, обучение школьников по спутниковым технологиям)
 • Президент с 19.06.2024 — Dr. Mengesha Ayene Ejigu (послание на сайте датировано 25.06.2024; более поздняя официальная страница не найдена)
 • Действует Дирекция внешних связей и партнёрств; в Telegram (окт. 2026) указан только gmail: bduexternalrelations@gmail.com; официального e-mail на сайте bdu.edu.et не найдено
 • Старые данные (IIE, 2023): директор внешних связей Dr. Manendante Mulugeta — актуальность не подтверждена
-• Почтовый ящик (P.O. Box) на сайте не подтверждён; основатели — при поддержке ЮНЕСКО и правительства СССР/России (упомянуто в послании президента)</t>
-        </is>
-      </c>
-      <c r="AH4" s="4" t="inlineStr">
+• Почтовый ящик (P.O. Box) на сайте не подтверждён; основатели — при поддержке ЮНЕСКО и правительства СССР/России (упомянуто в послании президента)
+• Рейтинги: Национального рейтинга с местами нет: МинОбр Эфиопии делит гос. вузы на категории (research / applied science / general), мест не публикует</t>
+        </is>
+      </c>
+      <c r="AI4" s="4" t="inlineStr">
         <is>
           <t>• Https://www.bdu.edu.et/
 • Https://www.bdu.edu.et/node/131
 • Https://www.bdu.edu.et/wagrl/
 • Https://bdu.edu.et/node/160
-• Https://t.me/s/bahir_dar_university</t>
-        </is>
-      </c>
-      <c r="AI4" s="4" t="inlineStr">
+• Https://t.me/s/bahir_dar_university
+https://figshare.com/articles/preprint/Ranking_Web_of_Universities_webometrics_info_July_2026_edition/33062150</t>
+        </is>
+      </c>
+      <c r="AJ4" s="4" t="inlineStr">
         <is>
           <t>2026-10-05</t>
         </is>
       </c>
-      <c r="AJ4" s="4" t="inlineStr"/>
+      <c r="AK4" s="4" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AJ4"/>
+  <autoFilter ref="A1:AK4"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1391,7 +1454,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AJ41"/>
+  <dimension ref="A1:AK41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1415,21 +1478,22 @@
     <col width="13" customWidth="1" min="19" max="19"/>
     <col width="13" customWidth="1" min="20" max="20"/>
     <col width="16" customWidth="1" min="21" max="21"/>
-    <col width="10" customWidth="1" min="22" max="22"/>
-    <col width="45" customWidth="1" min="23" max="23"/>
-    <col width="30" customWidth="1" min="24" max="24"/>
+    <col width="16" customWidth="1" min="22" max="22"/>
+    <col width="10" customWidth="1" min="23" max="23"/>
+    <col width="45" customWidth="1" min="24" max="24"/>
     <col width="30" customWidth="1" min="25" max="25"/>
-    <col width="40" customWidth="1" min="26" max="26"/>
-    <col width="45" customWidth="1" min="27" max="27"/>
-    <col width="22" customWidth="1" min="28" max="28"/>
-    <col width="11" customWidth="1" min="29" max="29"/>
-    <col width="9" customWidth="1" min="30" max="30"/>
-    <col width="12" customWidth="1" min="31" max="31"/>
-    <col width="11" customWidth="1" min="32" max="32"/>
-    <col width="55" customWidth="1" min="33" max="33"/>
-    <col width="60" customWidth="1" min="34" max="34"/>
-    <col width="12" customWidth="1" min="35" max="35"/>
-    <col width="24" customWidth="1" min="36" max="36"/>
+    <col width="30" customWidth="1" min="26" max="26"/>
+    <col width="40" customWidth="1" min="27" max="27"/>
+    <col width="45" customWidth="1" min="28" max="28"/>
+    <col width="22" customWidth="1" min="29" max="29"/>
+    <col width="11" customWidth="1" min="30" max="30"/>
+    <col width="9" customWidth="1" min="31" max="31"/>
+    <col width="12" customWidth="1" min="32" max="32"/>
+    <col width="11" customWidth="1" min="33" max="33"/>
+    <col width="55" customWidth="1" min="34" max="34"/>
+    <col width="60" customWidth="1" min="35" max="35"/>
+    <col width="12" customWidth="1" min="36" max="36"/>
+    <col width="24" customWidth="1" min="37" max="37"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1540,75 +1604,80 @@
       </c>
       <c r="V1" s="3" t="inlineStr">
         <is>
+          <t>Рейтинг Webometrics (мир)</t>
+        </is>
+      </c>
+      <c r="W1" s="3" t="inlineStr">
+        <is>
           <t>Запущено КА (спутников)</t>
         </is>
       </c>
-      <c r="W1" s="3" t="inlineStr">
+      <c r="X1" s="3" t="inlineStr">
         <is>
           <t>Названия запущенных КА (год)</t>
         </is>
       </c>
-      <c r="X1" s="3" t="inlineStr">
+      <c r="Y1" s="3" t="inlineStr">
         <is>
           <t>КА в разработке</t>
         </is>
       </c>
-      <c r="Y1" s="3" t="inlineStr">
+      <c r="Z1" s="3" t="inlineStr">
         <is>
           <t>Наземная станция</t>
         </is>
       </c>
-      <c r="Z1" s="3" t="inlineStr">
+      <c r="AA1" s="3" t="inlineStr">
         <is>
           <t>Космические подразделения</t>
         </is>
       </c>
-      <c r="AA1" s="3" t="inlineStr">
+      <c r="AB1" s="3" t="inlineStr">
         <is>
           <t>Партнёрства в космической сфере</t>
         </is>
       </c>
-      <c r="AB1" s="3" t="inlineStr">
+      <c r="AC1" s="3" t="inlineStr">
         <is>
           <t>Санкционные / ограничительные списки (США)</t>
         </is>
       </c>
-      <c r="AC1" s="3" t="inlineStr">
+      <c r="AD1" s="3" t="inlineStr">
         <is>
           <t>Космический индекс (0–100)</t>
         </is>
       </c>
-      <c r="AD1" s="3" t="inlineStr">
+      <c r="AE1" s="3" t="inlineStr">
         <is>
           <t>Волна рассылки</t>
         </is>
       </c>
-      <c r="AE1" s="3" t="inlineStr">
+      <c r="AF1" s="3" t="inlineStr">
         <is>
           <t>Проверка домена e-mail (MX)</t>
         </is>
       </c>
-      <c r="AF1" s="3" t="inlineStr">
+      <c r="AG1" s="3" t="inlineStr">
         <is>
           <t>Достоверность</t>
         </is>
       </c>
-      <c r="AG1" s="3" t="inlineStr">
+      <c r="AH1" s="3" t="inlineStr">
         <is>
           <t>Примечания</t>
         </is>
       </c>
-      <c r="AH1" s="3" t="inlineStr">
+      <c r="AI1" s="3" t="inlineStr">
         <is>
           <t>Источники</t>
         </is>
       </c>
-      <c r="AI1" s="3" t="inlineStr">
+      <c r="AJ1" s="3" t="inlineStr">
         <is>
           <t>Дата проверки</t>
         </is>
       </c>
-      <c r="AJ1" s="3" t="inlineStr">
+      <c r="AK1" s="3" t="inlineStr">
         <is>
           <t>Секретарь парткома (справочно, Китай)</t>
         </is>
@@ -1710,31 +1779,48 @@
           <t>Director General</t>
         </is>
       </c>
-      <c r="S2" s="4" t="inlineStr"/>
-      <c r="T2" s="4" t="inlineStr"/>
-      <c r="U2" s="4" t="inlineStr"/>
-      <c r="V2" s="4" t="n">
+      <c r="S2" s="4" t="inlineStr">
+        <is>
+          <t>QS2027: не в рейтинге</t>
+        </is>
+      </c>
+      <c r="T2" s="4" t="inlineStr">
+        <is>
+          <t>THE2027: не в рейтинге</t>
+        </is>
+      </c>
+      <c r="U2" s="4" t="inlineStr">
+        <is>
+          <t>нет общенационального рейтинга</t>
+        </is>
+      </c>
+      <c r="V2" s="4" t="inlineStr">
+        <is>
+          <t>нет в опубл. списке</t>
+        </is>
+      </c>
+      <c r="W2" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="W2" s="4" t="inlineStr">
+      <c r="X2" s="4" t="inlineStr">
         <is>
           <t>• ETRSS-1 (2019)
 • ET-SMART-RSS (2020)</t>
         </is>
       </c>
-      <c r="X2" s="4" t="inlineStr">
+      <c r="Y2" s="4" t="inlineStr">
         <is>
           <t>• ETRSS-2 (0.5 m EO satellite, joint development with Shanghai Engineering Center for Microsatellites
 • Launch planned Dec 2026)
 • Domestic satellite AIT centre planned with Roscosmos support</t>
         </is>
       </c>
-      <c r="Y2" s="4" t="inlineStr">
+      <c r="Z2" s="4" t="inlineStr">
         <is>
           <t>Multi-satellite tracking and data-receiving ground station at Entoto (installed May 2021; offered as paid data-reception service); 12-m EO satellite data receiving ground station (built 2024)</t>
         </is>
       </c>
-      <c r="Z2" s="4" t="inlineStr">
+      <c r="AA2" s="4" t="inlineStr">
         <is>
           <t>• Entoto Observatory and Research Center (EORC)
 • Satellite operations/space engineering directorates
@@ -1742,7 +1828,7 @@
 • Postgraduate programs in Astronomy &amp; Astrophysics, Space &amp; Planetary Science, Remote Sensing, Geodesy</t>
         </is>
       </c>
-      <c r="AA2" s="4" t="inlineStr">
+      <c r="AB2" s="4" t="inlineStr">
         <is>
           <t>• Shanghai Engineering Center for Microsatellites (ETRSS-2 contract, Nov 2024)
 • Beijing Smart Satellite Technology (ET-SMART-RSS)
@@ -1752,35 +1838,36 @@
 • FDRE Air Force (agreement)</t>
         </is>
       </c>
-      <c r="AB2" s="4" t="inlineStr"/>
-      <c r="AC2" s="4" t="n">
+      <c r="AC2" s="4" t="inlineStr"/>
+      <c r="AD2" s="4" t="n">
         <v>90</v>
       </c>
-      <c r="AD2" s="5" t="inlineStr">
+      <c r="AE2" s="5" t="inlineStr">
         <is>
           <t>1A</t>
         </is>
       </c>
-      <c r="AE2" s="4" t="inlineStr">
+      <c r="AF2" s="4" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="AF2" s="4" t="inlineStr">
+      <c r="AG2" s="4" t="inlineStr">
         <is>
           <t>высокая</t>
         </is>
       </c>
-      <c r="AG2" s="4" t="inlineStr">
+      <c r="AH2" s="4" t="inlineStr">
         <is>
           <t>• Национальное космическое агентство Эфиопии (бывш. ESSTI + EGII, объединены в 2022); ключевой адресат для созвездия
 • ETRSS-1 (2019) и ET-SMART-RSS (2020) построены в кооперации с Китаем; по данным ENA (янв. 2026) оба завершили срок службы
 • Адрес partnerships@ssgi.gov.et указан на сайте как контакт службы промышленного сотрудничества и партнёрств; отдельного международного отдела на сайте не найдено
 • Написание имени: Abdissa Yilma (сайт SSGI) / Abdisa Yilma (СМИ); на сайте SSGI указан как PhD, Fana пишет 'Mr.'
-• Идут переговоры с Роскосмосом о центре сборки/испытаний спутников (апр. 2026) — благоприятный контекст для БРИКС-сотрудничества</t>
-        </is>
-      </c>
-      <c r="AH2" s="4" t="inlineStr">
+• Идут переговоры с Роскосмосом о центре сборки/испытаний спутников (апр. 2026) — благоприятный контекст для БРИКС-сотрудничества
+• Рейтинги: Национального рейтинга с местами нет: МинОбр Эфиопии делит гос. вузы на категории (research / applied science / general), мест не публикует</t>
+        </is>
+      </c>
+      <c r="AI2" s="4" t="inlineStr">
         <is>
           <t>• Https://ssgi.gov.et
 • Https://ssgi.gov.et/assets/index-CddNteli.js (site leadership/contact data)
@@ -1791,12 +1878,12 @@
 • Nanosats.csv</t>
         </is>
       </c>
-      <c r="AI2" s="4" t="inlineStr">
+      <c r="AJ2" s="4" t="inlineStr">
         <is>
           <t>2026-10-05</t>
         </is>
       </c>
-      <c r="AJ2" s="4" t="inlineStr"/>
+      <c r="AK2" s="4" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
@@ -1895,70 +1982,90 @@
           <t>President</t>
         </is>
       </c>
-      <c r="S3" s="4" t="inlineStr"/>
-      <c r="T3" s="4" t="inlineStr"/>
-      <c r="U3" s="4" t="inlineStr"/>
-      <c r="V3" s="4" t="n">
+      <c r="S3" s="4" t="inlineStr">
+        <is>
+          <t>QS2027: 951–1000</t>
+        </is>
+      </c>
+      <c r="T3" s="4" t="inlineStr">
+        <is>
+          <t>THE2027: не в рейтинге</t>
+        </is>
+      </c>
+      <c r="U3" s="4" t="inlineStr">
+        <is>
+          <t>нет общенационального рейтинга</t>
+        </is>
+      </c>
+      <c r="V3" s="4" t="inlineStr">
+        <is>
+          <t>1109</t>
+        </is>
+      </c>
+      <c r="W3" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="W3" s="4" t="inlineStr"/>
-      <c r="X3" s="4" t="inlineStr">
+      <c r="X3" s="4" t="inlineStr"/>
+      <c r="Y3" s="4" t="inlineStr">
         <is>
           <t>ET-SAT (2U CubeSat by AAiT, pre-selected for QB50) — cancelled, never launched</t>
         </is>
       </c>
-      <c r="Y3" s="4" t="inlineStr"/>
-      <c r="Z3" s="4" t="inlineStr">
+      <c r="Z3" s="4" t="inlineStr"/>
+      <c r="AA3" s="4" t="inlineStr">
         <is>
           <t>• Department of Physics (astrophysics / astronomy research stream)
 • Addis Ababa Institute of Technology — School of Electrical &amp; Computer Engineering (ELEDIA@AAiT research group, communication engineering)</t>
         </is>
       </c>
-      <c r="AA3" s="4" t="inlineStr"/>
       <c r="AB3" s="4" t="inlineStr"/>
-      <c r="AC3" s="4" t="n">
-        <v>25</v>
-      </c>
-      <c r="AD3" s="6" t="inlineStr">
+      <c r="AC3" s="4" t="inlineStr"/>
+      <c r="AD3" s="4" t="n">
+        <v>31</v>
+      </c>
+      <c r="AE3" s="6" t="inlineStr">
         <is>
           <t>1B</t>
         </is>
       </c>
-      <c r="AE3" s="4" t="inlineStr">
+      <c r="AF3" s="4" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="AF3" s="4" t="inlineStr">
+      <c r="AG3" s="4" t="inlineStr">
         <is>
           <t>средняя</t>
         </is>
       </c>
-      <c r="AG3" s="4" t="inlineStr">
+      <c r="AH3" s="4" t="inlineStr">
         <is>
           <t>• Ведущий университет страны; сайт aau.edu.et — JS-приложение, данные взяты из официального API api.aau.edu.et
 • Международными связями ведает Office of Partnerships (подразделение AAU Global) при вице-президенте по партнёрству и коммуникациям; по ENA (фев. 2025) этот пост занимала Dr. Rahel Argaw, в текущем списке руководства на сайте её нет — не подтверждено на 2026
 • Отдельного e-mail президента не опубликовано; email_general — Office of Communication (также в офисе президента, 6 Kilo)
 • QS 2026: 851–900 (fsxbusiness); значение QS 2027 (по поисковой выдаче 951–1000) не подтверждено с открытой страницы — поле оставлено пустым. В THE 2027 по входным данным не ранжирован
-• Спутник ET-SAT (AAiT, QB50) отменён; запусков нет. Почтовый ящик P.O. Box 1176 подтверждён для подразделения AAU (ACEWM), общеуниверситетский P.O. Box стоит перепроверить</t>
-        </is>
-      </c>
-      <c r="AH3" s="4" t="inlineStr">
+• Спутник ET-SAT (AAiT, QB50) отменён; запусков нет. Почтовый ящик P.O. Box 1176 подтверждён для подразделения AAU (ACEWM), общеуниверситетский P.O. Box стоит перепроверить
+• Рейтинги: Национального рейтинга с местами нет: МинОбр Эфиопии делит гос. вузы на категории (research / applied science / general), мест не публикует</t>
+        </is>
+      </c>
+      <c r="AI3" s="4" t="inlineStr">
         <is>
           <t>• Https://api.aau.edu.et/leaderships/
 • Https://api.aau.edu.et/contents/ (Office of Partnerships &amp; Office of Communication pages, updated 2026-04-21)
 • Https://www.ena.et/web/eng/w/eng_6063594
 • Https://www.fsxbusiness.com/aau-tops-east-africa-in-qs-rankings
 • Https://www.nanosats.eu/sat/et-sat
-• Nanosats.csv</t>
-        </is>
-      </c>
-      <c r="AI3" s="4" t="inlineStr">
+• Nanosats.csv
+https://www.topuniversities.com/world-university-rankings (QS WUR 2027)
+https://figshare.com/articles/preprint/Ranking_Web_of_Universities_webometrics_info_July_2026_edition/33062150</t>
+        </is>
+      </c>
+      <c r="AJ3" s="4" t="inlineStr">
         <is>
           <t>2026-10-05</t>
         </is>
       </c>
-      <c r="AJ3" s="4" t="inlineStr"/>
+      <c r="AK3" s="4" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
@@ -2057,65 +2164,84 @@
           <t>President</t>
         </is>
       </c>
-      <c r="S4" s="4" t="inlineStr"/>
-      <c r="T4" s="4" t="inlineStr"/>
-      <c r="U4" s="4" t="inlineStr"/>
-      <c r="V4" s="4" t="n">
+      <c r="S4" s="4" t="inlineStr">
+        <is>
+          <t>QS2027: не в рейтинге</t>
+        </is>
+      </c>
+      <c r="T4" s="4" t="inlineStr">
+        <is>
+          <t>THE2027: не в рейтинге</t>
+        </is>
+      </c>
+      <c r="U4" s="4" t="inlineStr">
+        <is>
+          <t>нет общенационального рейтинга</t>
+        </is>
+      </c>
+      <c r="V4" s="4" t="inlineStr">
+        <is>
+          <t>3527</t>
+        </is>
+      </c>
+      <c r="W4" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="W4" s="4" t="inlineStr"/>
       <c r="X4" s="4" t="inlineStr"/>
       <c r="Y4" s="4" t="inlineStr"/>
-      <c r="Z4" s="4" t="inlineStr">
+      <c r="Z4" s="4" t="inlineStr"/>
+      <c r="AA4" s="4" t="inlineStr">
         <is>
           <t>Joint Aerospace Engineering Postgraduate Program with SSGI (M.Sc. Space Engineering, M.Sc. Aeronautical Engineering — drones, CubeSats, rockets)</t>
         </is>
       </c>
-      <c r="AA4" s="4" t="inlineStr">
+      <c r="AB4" s="4" t="inlineStr">
         <is>
           <t>Space Science and Geospatial Institute (SSGI) — joint aerospace postgraduate program</t>
         </is>
       </c>
-      <c r="AB4" s="4" t="inlineStr"/>
-      <c r="AC4" s="4" t="n">
+      <c r="AC4" s="4" t="inlineStr"/>
+      <c r="AD4" s="4" t="n">
         <v>20</v>
       </c>
-      <c r="AD4" s="7" t="inlineStr">
+      <c r="AE4" s="7" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="AE4" s="4" t="inlineStr">
+      <c r="AF4" s="4" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="AF4" s="4" t="inlineStr">
+      <c r="AG4" s="4" t="inlineStr">
         <is>
           <t>высокая</t>
         </is>
       </c>
-      <c r="AG4" s="4" t="inlineStr">
+      <c r="AH4" s="4" t="inlineStr">
         <is>
           <t>• Спутников на орбите не найдено; совместная магистратура по аэрокосмической инженерии с SSGI (включая CubeSat) — хорошая точка входа
 • Телефон +251 11 462 4178 найден в исходном коде страницы офиса президента (не отображается на странице) — проверить
-• Альтернативный личный адрес директора: biniam.atnafe@aastu.edu.et; моб. +251 911 995 069; директор офиса президента — Solomon Molla Alemu (PhD), po.director@aastu.edu.et</t>
-        </is>
-      </c>
-      <c r="AH4" s="4" t="inlineStr">
+• Альтернативный личный адрес директора: biniam.atnafe@aastu.edu.et; моб. +251 911 995 069; директор офиса президента — Solomon Molla Alemu (PhD), po.director@aastu.edu.et
+• Рейтинги: Национального рейтинга с местами нет: МинОбр Эфиопии делит гос. вузы на категории (research / applied science / general), мест не публикует</t>
+        </is>
+      </c>
+      <c r="AI4" s="4" t="inlineStr">
         <is>
           <t>• Https://www.aastu.edu.et/
 • Https://www.aastu.edu.et/president-office/
 • Https://www.aastu.edu.et/international-relations-and-partnerships/
-• Https://ssgi.gov.et/api/api/news (Aerospace Engineering Postgraduate Program)</t>
-        </is>
-      </c>
-      <c r="AI4" s="4" t="inlineStr">
+• Https://ssgi.gov.et/api/api/news (Aerospace Engineering Postgraduate Program)
+https://figshare.com/articles/preprint/Ranking_Web_of_Universities_webometrics_info_July_2026_edition/33062150</t>
+        </is>
+      </c>
+      <c r="AJ4" s="4" t="inlineStr">
         <is>
           <t>2026-10-05</t>
         </is>
       </c>
-      <c r="AJ4" s="4" t="inlineStr"/>
+      <c r="AK4" s="4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
@@ -2210,70 +2336,89 @@
           <t>President</t>
         </is>
       </c>
-      <c r="S5" s="4" t="inlineStr"/>
-      <c r="T5" s="4" t="inlineStr"/>
-      <c r="U5" s="4" t="inlineStr"/>
-      <c r="V5" s="4" t="n">
+      <c r="S5" s="4" t="inlineStr">
+        <is>
+          <t>QS2027: не в рейтинге</t>
+        </is>
+      </c>
+      <c r="T5" s="4" t="inlineStr">
+        <is>
+          <t>THE2027: не в рейтинге</t>
+        </is>
+      </c>
+      <c r="U5" s="4" t="inlineStr">
+        <is>
+          <t>нет общенационального рейтинга</t>
+        </is>
+      </c>
+      <c r="V5" s="4" t="inlineStr">
+        <is>
+          <t>2237</t>
+        </is>
+      </c>
+      <c r="W5" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="W5" s="4" t="inlineStr"/>
       <c r="X5" s="4" t="inlineStr"/>
-      <c r="Y5" s="4" t="inlineStr">
+      <c r="Y5" s="4" t="inlineStr"/>
+      <c r="Z5" s="4" t="inlineStr">
         <is>
           <t>Blue Nile Radar (BNR) / geospace radar facilities of the Washera Geospace and Radar Science Laboratory</t>
         </is>
       </c>
-      <c r="Z5" s="4" t="inlineStr">
+      <c r="AA5" s="4" t="inlineStr">
         <is>
           <t>• Washera Geospace and Radar Science Laboratory (WaGRL, College of Science)
 • Geospatial Data &amp; Technology Center
 • Bahir Dar Institute of Technology</t>
         </is>
       </c>
-      <c r="AA5" s="4" t="inlineStr"/>
       <c r="AB5" s="4" t="inlineStr"/>
-      <c r="AC5" s="4" t="n">
+      <c r="AC5" s="4" t="inlineStr"/>
+      <c r="AD5" s="4" t="n">
         <v>20</v>
       </c>
-      <c r="AD5" s="6" t="inlineStr">
+      <c r="AE5" s="6" t="inlineStr">
         <is>
           <t>1B</t>
         </is>
       </c>
-      <c r="AE5" s="4" t="inlineStr">
+      <c r="AF5" s="4" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="AF5" s="4" t="inlineStr">
+      <c r="AG5" s="4" t="inlineStr">
         <is>
           <t>средняя</t>
         </is>
       </c>
-      <c r="AG5" s="4" t="inlineStr">
+      <c r="AH5" s="4" t="inlineStr">
         <is>
           <t>• Спутников на орбите не найдено; есть лаборатория геокосмоса и радаров (ионосфера, TEC-модели, обучение школьников по спутниковым технологиям)
 • Президент с 19.06.2024 — Dr. Mengesha Ayene Ejigu (послание на сайте датировано 25.06.2024; более поздняя официальная страница не найдена)
 • Действует Дирекция внешних связей и партнёрств; в Telegram (окт. 2026) указан только gmail: bduexternalrelations@gmail.com; официального e-mail на сайте bdu.edu.et не найдено
 • Старые данные (IIE, 2023): директор внешних связей Dr. Manendante Mulugeta — актуальность не подтверждена
-• Почтовый ящик (P.O. Box) на сайте не подтверждён; основатели — при поддержке ЮНЕСКО и правительства СССР/России (упомянуто в послании президента)</t>
-        </is>
-      </c>
-      <c r="AH5" s="4" t="inlineStr">
+• Почтовый ящик (P.O. Box) на сайте не подтверждён; основатели — при поддержке ЮНЕСКО и правительства СССР/России (упомянуто в послании президента)
+• Рейтинги: Национального рейтинга с местами нет: МинОбр Эфиопии делит гос. вузы на категории (research / applied science / general), мест не публикует</t>
+        </is>
+      </c>
+      <c r="AI5" s="4" t="inlineStr">
         <is>
           <t>• Https://www.bdu.edu.et/
 • Https://www.bdu.edu.et/node/131
 • Https://www.bdu.edu.et/wagrl/
 • Https://bdu.edu.et/node/160
-• Https://t.me/s/bahir_dar_university</t>
-        </is>
-      </c>
-      <c r="AI5" s="4" t="inlineStr">
+• Https://t.me/s/bahir_dar_university
+https://figshare.com/articles/preprint/Ranking_Web_of_Universities_webometrics_info_July_2026_edition/33062150</t>
+        </is>
+      </c>
+      <c r="AJ5" s="4" t="inlineStr">
         <is>
           <t>2026-10-05</t>
         </is>
       </c>
-      <c r="AJ5" s="4" t="inlineStr"/>
+      <c r="AK5" s="4" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
@@ -2373,63 +2518,82 @@
           <t>President</t>
         </is>
       </c>
-      <c r="S6" s="4" t="inlineStr"/>
-      <c r="T6" s="4" t="inlineStr"/>
-      <c r="U6" s="4" t="inlineStr"/>
-      <c r="V6" s="4" t="n">
+      <c r="S6" s="4" t="inlineStr">
+        <is>
+          <t>QS2027: не в рейтинге</t>
+        </is>
+      </c>
+      <c r="T6" s="4" t="inlineStr">
+        <is>
+          <t>THE2027: не в рейтинге</t>
+        </is>
+      </c>
+      <c r="U6" s="4" t="inlineStr">
+        <is>
+          <t>нет общенационального рейтинга</t>
+        </is>
+      </c>
+      <c r="V6" s="4" t="inlineStr">
+        <is>
+          <t>3948</t>
+        </is>
+      </c>
+      <c r="W6" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="W6" s="4" t="inlineStr"/>
       <c r="X6" s="4" t="inlineStr"/>
       <c r="Y6" s="4" t="inlineStr"/>
       <c r="Z6" s="4" t="inlineStr"/>
-      <c r="AA6" s="4" t="inlineStr">
+      <c r="AA6" s="4" t="inlineStr"/>
+      <c r="AB6" s="4" t="inlineStr">
         <is>
           <t>Space Science and Geospatial Institute (SSGI) — agreement Apr 2024 on ASTU consultancy for the ETRSS-2 Earth-observation satellite project</t>
         </is>
       </c>
-      <c r="AB6" s="4" t="inlineStr"/>
-      <c r="AC6" s="4" t="n">
+      <c r="AC6" s="4" t="inlineStr"/>
+      <c r="AD6" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="AD6" s="8" t="inlineStr">
+      <c r="AE6" s="8" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="AE6" s="4" t="inlineStr">
+      <c r="AF6" s="4" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="AF6" s="4" t="inlineStr">
+      <c r="AG6" s="4" t="inlineStr">
         <is>
           <t>высокая</t>
         </is>
       </c>
-      <c r="AG6" s="4" t="inlineStr">
+      <c r="AH6" s="4" t="inlineStr">
         <is>
           <t>• Ведущий технический университет (одобрен как university of science and technology); соглашение с SSGI по проекту спутника ETRSS-2 (2024) — хороший контекст
 • Email_international — личный адрес директора Office of Internationalization and Partnership (страница обновлена фев. 2025); альтернативы: irccd@astu.edu.et (International Relations and Corporate Communications, контакт в подвале сайта) и pireo@astu.edu.et (Public and International Relations Executive, Mr. Girma Megersa Bedane)
 • Отдельный e-mail президента не опубликован; Chief Executive Officer of President Office — Dr. Worku Jifara Sori
-• В QS 2027 и THE 2027 не найден</t>
-        </is>
-      </c>
-      <c r="AH6" s="4" t="inlineStr">
+• В QS 2027 и THE 2027 не найден
+• Рейтинги: Национального рейтинга с местами нет: МинОбр Эфиопии делит гос. вузы на категории (research / applied science / general), мест не публикует</t>
+        </is>
+      </c>
+      <c r="AI6" s="4" t="inlineStr">
         <is>
           <t>• Https://www.astu.edu.et
 • Https://www.astu.edu.et/offices/president-office/president-offices
 • Https://www.astu.edu.et/offices/president-office/internationalization-for-research-and-partnership
 • Https://www.astu.edu.et/offices/president-office/public-and-international-relations
-• Http://spaceinafrica.com/2024/04/11/ssgi-signs-agreement-with-adama-science-and-technology-university/</t>
-        </is>
-      </c>
-      <c r="AI6" s="4" t="inlineStr">
+• Http://spaceinafrica.com/2024/04/11/ssgi-signs-agreement-with-adama-science-and-technology-university/
+https://figshare.com/articles/preprint/Ranking_Web_of_Universities_webometrics_info_July_2026_edition/33062150</t>
+        </is>
+      </c>
+      <c r="AJ6" s="4" t="inlineStr">
         <is>
           <t>2026-10-05</t>
         </is>
       </c>
-      <c r="AJ6" s="4" t="inlineStr"/>
+      <c r="AK6" s="4" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
@@ -2523,49 +2687,67 @@
           <t>President</t>
         </is>
       </c>
-      <c r="S7" s="4" t="inlineStr"/>
-      <c r="T7" s="4" t="inlineStr"/>
-      <c r="U7" s="4" t="inlineStr"/>
-      <c r="V7" s="4" t="n">
+      <c r="S7" s="4" t="inlineStr">
+        <is>
+          <t>QS2027: не в рейтинге</t>
+        </is>
+      </c>
+      <c r="T7" s="4" t="inlineStr">
+        <is>
+          <t>THE2027: не в рейтинге</t>
+        </is>
+      </c>
+      <c r="U7" s="4" t="inlineStr">
+        <is>
+          <t>нет общенационального рейтинга</t>
+        </is>
+      </c>
+      <c r="V7" s="4" t="inlineStr">
+        <is>
+          <t>нет в опубл. списке</t>
+        </is>
+      </c>
+      <c r="W7" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="W7" s="4" t="inlineStr"/>
       <c r="X7" s="4" t="inlineStr"/>
       <c r="Y7" s="4" t="inlineStr"/>
       <c r="Z7" s="4" t="inlineStr"/>
-      <c r="AA7" s="4" t="inlineStr">
+      <c r="AA7" s="4" t="inlineStr"/>
+      <c r="AB7" s="4" t="inlineStr">
         <is>
           <t>Boeing (STEM School Program, 4th edition 2026)</t>
         </is>
       </c>
-      <c r="AB7" s="4" t="inlineStr"/>
-      <c r="AC7" s="4" t="n">
+      <c r="AC7" s="4" t="inlineStr"/>
+      <c r="AD7" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="AD7" s="8" t="inlineStr">
+      <c r="AE7" s="8" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="AE7" s="4" t="inlineStr">
+      <c r="AF7" s="4" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="AF7" s="4" t="inlineStr">
+      <c r="AG7" s="4" t="inlineStr">
         <is>
           <t>средняя</t>
         </is>
       </c>
-      <c r="AG7" s="4" t="inlineStr">
+      <c r="AH7" s="4" t="inlineStr">
         <is>
           <t>• Корпоративный университет авиакомпании Ethiopian Airlines Group (госкомпания), бывшая Ethiopian Aviation Academy; поле ownership условно — 'агентство/госпредприятие', не Минобразования
 • Профильно близок к аэрокосмической тематике (техобслуживание ВС, УВД, тренажёры) — перспективный партнёр, хотя спутниковых проектов не найдено
 • Отдельного международного офиса и его e-mail не опубликовано; общие адреса: InfoEAU@eau.edu.et и etauinfo@ethiopianairlines.com; страница руководства на сайте пока пустая
-• Почтовый адрес/P.O. Box на сайте не найден (кампус в Аддис-Абебе)</t>
-        </is>
-      </c>
-      <c r="AH7" s="4" t="inlineStr">
+• Почтовый адрес/P.O. Box на сайте не найден (кампус в Аддис-Абебе)
+• Рейтинги: Национального рейтинга с местами нет: МинОбр Эфиопии делит гос. вузы на категории (research / applied science / general), мест не публикует</t>
+        </is>
+      </c>
+      <c r="AI7" s="4" t="inlineStr">
         <is>
           <t>• Https://www.eau.edu.et
 • Https://eau.edu.et/about/news
@@ -2575,12 +2757,12 @@
 • Nanosats.csv (nation=Ethiopia: only ESSTI ET-SMART-RSS and cancelled AAiT ET-SAT)</t>
         </is>
       </c>
-      <c r="AI7" s="4" t="inlineStr">
+      <c r="AJ7" s="4" t="inlineStr">
         <is>
           <t>2026-10-05</t>
         </is>
       </c>
-      <c r="AJ7" s="4" t="inlineStr"/>
+      <c r="AK7" s="4" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
@@ -2679,50 +2861,64 @@
           <t>President</t>
         </is>
       </c>
-      <c r="S8" s="4" t="inlineStr"/>
+      <c r="S8" s="4" t="inlineStr">
+        <is>
+          <t>QS2027: не в рейтинге</t>
+        </is>
+      </c>
       <c r="T8" s="4" t="inlineStr">
         <is>
           <t>THE2027: 1201–1400</t>
         </is>
       </c>
-      <c r="U8" s="4" t="inlineStr"/>
-      <c r="V8" s="4" t="n">
+      <c r="U8" s="4" t="inlineStr">
+        <is>
+          <t>нет общенационального рейтинга</t>
+        </is>
+      </c>
+      <c r="V8" s="4" t="inlineStr">
+        <is>
+          <t>3375</t>
+        </is>
+      </c>
+      <c r="W8" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="W8" s="4" t="inlineStr"/>
       <c r="X8" s="4" t="inlineStr"/>
       <c r="Y8" s="4" t="inlineStr"/>
       <c r="Z8" s="4" t="inlineStr"/>
       <c r="AA8" s="4" t="inlineStr"/>
       <c r="AB8" s="4" t="inlineStr"/>
-      <c r="AC8" s="4" t="n">
+      <c r="AC8" s="4" t="inlineStr"/>
+      <c r="AD8" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="AD8" s="8" t="inlineStr">
+      <c r="AE8" s="8" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="AE8" s="4" t="inlineStr">
+      <c r="AF8" s="4" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="AF8" s="4" t="inlineStr">
+      <c r="AG8" s="4" t="inlineStr">
         <is>
           <t>средняя</t>
         </is>
       </c>
-      <c r="AG8" s="4" t="inlineStr">
+      <c r="AH8" s="4" t="inlineStr">
         <is>
           <t>• ВНИМАНИЕ: Тыграй. С 9 сент. 2026 Минобразования (министр Prof. Berhanu Nega) приостановило зачисление новых студентов в 4 университета Тыграя (Мэкэле, Аксум, Адыграт, Райя) и временно переводит их студентов в другие вузы из-за небезопасности; часть кампусов (Kuha campus MU) используется для размещения раненых военных. MU заявляет, что 6 из 7 кампусов работают
 • Президент Dr. Fana Hagos Berhane (с апр. 2021) — в 2026 стала членом International Advisory Committee китайского China–BRICS New Era Science and Technology Innovation Incubation Park: очень благоприятный контекст для БРИКС-приглашения
 • На сайте указан Provost for International Affairs and Global Collaboration — Dr. Shi Yongsheng (provost.office@mu.edu.et) — возможный дополнительный адресат
 • Имя директора International Affairs Directorate на сайте не указано; адрес ia.director@mu.edu.et, тел. +251-344-410976, Ground Floor, Room A1-114
-• Космических проектов/спутников не найдено</t>
-        </is>
-      </c>
-      <c r="AH8" s="4" t="inlineStr">
+• Космических проектов/спутников не найдено
+• Рейтинги: Национального рейтинга с местами нет: МинОбр Эфиопии делит гос. вузы на категории (research / applied science / general), мест не публикует</t>
+        </is>
+      </c>
+      <c r="AI8" s="4" t="inlineStr">
         <is>
           <t>• Https://www.mu.edu.et
 • Https://www.mu.edu.et/index.php/about (MU Contacts)
@@ -2731,15 +2927,17 @@
 • Https://www.mu.edu.et/index.php/news/new-international-scientific-appointment
 • Https://www.riotimesonline.com/ethiopia-tigray-university-students-reassigned-2026/
 • Https://addisstandard.com/mekelle-university-asks-education-ministry-to-assign-students-says-six-of-its-seven-campuses-remain-operational/
-• THE 2027 (input)</t>
-        </is>
-      </c>
-      <c r="AI8" s="4" t="inlineStr">
+• THE 2027 (input)
+https://www.timeshighereducation.com/world-university-rankings/2027/world-ranking
+https://figshare.com/articles/preprint/Ranking_Web_of_Universities_webometrics_info_July_2026_edition/33062150</t>
+        </is>
+      </c>
+      <c r="AJ8" s="4" t="inlineStr">
         <is>
           <t>2026-10-05</t>
         </is>
       </c>
-      <c r="AJ8" s="4" t="inlineStr"/>
+      <c r="AK8" s="4" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
@@ -2806,54 +3004,64 @@
           <t>President</t>
         </is>
       </c>
-      <c r="S9" s="4" t="inlineStr"/>
-      <c r="T9" s="4" t="inlineStr"/>
+      <c r="S9" s="4" t="inlineStr">
+        <is>
+          <t>QS2027: не в рейтинге</t>
+        </is>
+      </c>
+      <c r="T9" s="4" t="inlineStr">
+        <is>
+          <t>THE2027: не в рейтинге</t>
+        </is>
+      </c>
       <c r="U9" s="4" t="inlineStr"/>
-      <c r="V9" s="4" t="n">
+      <c r="V9" s="4" t="inlineStr"/>
+      <c r="W9" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="W9" s="4" t="inlineStr"/>
       <c r="X9" s="4" t="inlineStr"/>
       <c r="Y9" s="4" t="inlineStr"/>
       <c r="Z9" s="4" t="inlineStr"/>
       <c r="AA9" s="4" t="inlineStr"/>
       <c r="AB9" s="4" t="inlineStr"/>
-      <c r="AC9" s="4" t="n">
+      <c r="AC9" s="4" t="inlineStr"/>
+      <c r="AD9" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="AD9" s="8" t="inlineStr">
+      <c r="AE9" s="8" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="AE9" s="4" t="inlineStr"/>
-      <c r="AF9" s="4" t="inlineStr">
+      <c r="AF9" s="4" t="inlineStr"/>
+      <c r="AG9" s="4" t="inlineStr">
         <is>
           <t>низкая</t>
         </is>
       </c>
-      <c r="AG9" s="4" t="inlineStr">
+      <c r="AH9" s="4" t="inlineStr">
         <is>
           <t>• Спутников на орбите не найдено (проверка: nanosats.csv и поиск 'Ethiopian university CubeSat launched', окт. 2026)
 • Университет в Тыграе; сайт adu.edu.et недоступен (503 / сброс соединения, повторно 04.10.2026); e-mail и телефон не найдены
 • Президент Dr. Gebremichael Woldegabriel — по поисковой выдаче официального сайта (выпуск 524 студентов 20.06.2026, новости июля 2026); открытой страницей НЕ подтверждено
 • Перед рассылкой учесть ситуацию с доступом/связью в Тыграе
-• Перепроверка: Сайт adu.edu.et по-прежнему недоступен; президент Dr. Gebremichael Woldegabriel внесён по выдаче официальных новостей сайта (06–07.2026), страницы не открыты — контакты не найдены</t>
-        </is>
-      </c>
-      <c r="AH9" s="4" t="inlineStr">
+• Перепроверка: Сайт adu.edu.et по-прежнему недоступен; президент Dr. Gebremichael Woldegabriel внесён по выдаче официальных новостей сайта (06–07.2026), страницы не открыты — контакты не найдены
+• Ручная проверка: Рейтинги: QS 2027 — официальный файл данных topuniversities.com (qs-rankings-data/en/4153156.txt), сверка 05.10.2026; THE 2027 — список THE World University Rankings 2027 (data/sources/the2027.json). Webometrics: webometrics.info не открывается (DNS) — не заполнено</t>
+        </is>
+      </c>
+      <c r="AI9" s="4" t="inlineStr">
         <is>
           <t>• Https://adu.edu.et (HTTP 503 / unreachable, Oct 2026)
 • Https://adu.edu.et/2026/06/20/ (search index only)
 • Https://adu.edu.et/2026/06/20/ (snippet)</t>
         </is>
       </c>
-      <c r="AI9" s="4" t="inlineStr">
+      <c r="AJ9" s="4" t="inlineStr">
         <is>
           <t>2026-10-05</t>
         </is>
       </c>
-      <c r="AJ9" s="4" t="inlineStr"/>
+      <c r="AK9" s="4" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
@@ -2948,45 +3156,63 @@
           <t>President</t>
         </is>
       </c>
-      <c r="S10" s="4" t="inlineStr"/>
-      <c r="T10" s="4" t="inlineStr"/>
-      <c r="U10" s="4" t="inlineStr"/>
-      <c r="V10" s="4" t="n">
+      <c r="S10" s="4" t="inlineStr">
+        <is>
+          <t>QS2027: не в рейтинге</t>
+        </is>
+      </c>
+      <c r="T10" s="4" t="inlineStr">
+        <is>
+          <t>THE2027: не в рейтинге</t>
+        </is>
+      </c>
+      <c r="U10" s="4" t="inlineStr">
+        <is>
+          <t>нет общенационального рейтинга</t>
+        </is>
+      </c>
+      <c r="V10" s="4" t="inlineStr">
+        <is>
+          <t>нет в опубл. списке</t>
+        </is>
+      </c>
+      <c r="W10" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="W10" s="4" t="inlineStr"/>
       <c r="X10" s="4" t="inlineStr"/>
       <c r="Y10" s="4" t="inlineStr"/>
       <c r="Z10" s="4" t="inlineStr"/>
       <c r="AA10" s="4" t="inlineStr"/>
       <c r="AB10" s="4" t="inlineStr"/>
-      <c r="AC10" s="4" t="n">
+      <c r="AC10" s="4" t="inlineStr"/>
+      <c r="AD10" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="AD10" s="8" t="inlineStr">
+      <c r="AE10" s="8" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="AE10" s="4" t="inlineStr">
+      <c r="AF10" s="4" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="AF10" s="4" t="inlineStr">
+      <c r="AG10" s="4" t="inlineStr">
         <is>
           <t>средняя</t>
         </is>
       </c>
-      <c r="AG10" s="4" t="inlineStr">
+      <c r="AH10" s="4" t="inlineStr">
         <is>
           <t>• ВНИМАНИЕ: Тыграй. С 9 сент. 2026 МинОбр приостановило зачисление новых студентов и временно переводит студентов Аксумского университета в другие вузы (небезопасность; на главном кампусе размещены раненые военные). Руководство Аксума требовало отменить решение
 • Public and International Relations Executive — Mr. Teklay Gebremicheal Teklu (только gmail: teklaygt21@gmail.com / aksumuniversity2025@gmail.com, тел. +251 980 103 118); International Team Leader — Mr. Gebre Welejewergis (+251 914 494 622)
 • В подвале сайта ящик PIR опубликован обрезанным: 'PRD@mail.aku.edu.e' (вероятно PRD@mail.aku.edu.et, домен mail.aku.edu.et имеет MX Microsoft 365) — не подтверждён, поэтому письмо на info@mail.aku.edu.et
-• Номер P.O. Box на сайте не указан; спутниковых проектов не найдено</t>
-        </is>
-      </c>
-      <c r="AH10" s="4" t="inlineStr">
+• Номер P.O. Box на сайте не указан; спутниковых проектов не найдено
+• Рейтинги: Национального рейтинга с местами нет: МинОбр Эфиопии делит гос. вузы на категории (research / applied science / general), мест не публикует</t>
+        </is>
+      </c>
+      <c r="AI10" s="4" t="inlineStr">
         <is>
           <t>• Https://aku.edu.et
 • Https://aku.edu.et/contact-us/
@@ -2997,12 +3223,12 @@
 • Nanosats.csv (nation=Ethiopia: only ESSTI ET-SMART-RSS and cancelled AAiT ET-SAT)</t>
         </is>
       </c>
-      <c r="AI10" s="4" t="inlineStr">
+      <c r="AJ10" s="4" t="inlineStr">
         <is>
           <t>2026-10-05</t>
         </is>
       </c>
-      <c r="AJ10" s="4" t="inlineStr"/>
+      <c r="AK10" s="4" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
@@ -3061,53 +3287,63 @@
           <t>President</t>
         </is>
       </c>
-      <c r="S11" s="4" t="inlineStr"/>
-      <c r="T11" s="4" t="inlineStr"/>
+      <c r="S11" s="4" t="inlineStr">
+        <is>
+          <t>QS2027: не в рейтинге</t>
+        </is>
+      </c>
+      <c r="T11" s="4" t="inlineStr">
+        <is>
+          <t>THE2027: не в рейтинге</t>
+        </is>
+      </c>
       <c r="U11" s="4" t="inlineStr"/>
-      <c r="V11" s="4" t="n">
+      <c r="V11" s="4" t="inlineStr"/>
+      <c r="W11" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="W11" s="4" t="inlineStr"/>
       <c r="X11" s="4" t="inlineStr"/>
       <c r="Y11" s="4" t="inlineStr"/>
       <c r="Z11" s="4" t="inlineStr"/>
       <c r="AA11" s="4" t="inlineStr"/>
       <c r="AB11" s="4" t="inlineStr"/>
-      <c r="AC11" s="4" t="n">
+      <c r="AC11" s="4" t="inlineStr"/>
+      <c r="AD11" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="AD11" s="8" t="inlineStr">
+      <c r="AE11" s="8" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="AE11" s="4" t="inlineStr"/>
-      <c r="AF11" s="4" t="inlineStr">
+      <c r="AF11" s="4" t="inlineStr"/>
+      <c r="AG11" s="4" t="inlineStr">
         <is>
           <t>низкая</t>
         </is>
       </c>
-      <c r="AG11" s="4" t="inlineStr">
+      <c r="AH11" s="4" t="inlineStr">
         <is>
           <t>• Спутников на орбите не найдено (проверка: nanosats.csv и поиск 'Ethiopian university CubeSat launched', окт. 2026)
 • Сайт ambou.edu.et недоступен (ошибка базы данных HTTP 500 на всех страницах, 04.10.2026) — контакты не проверены
 • Поисковая выдача (на основе Википедии) называет президентом Dr. Bayissa Leta — НЕ подтверждено официальным источником, поле оставлено пустым
 • Нужна повторная проверка сайта позже: страницы president-message и president-office-head существуют в поисковом индексе
-• Перепроверка: Сайт ambou.edu.et недоступен (ERR_ADDRESS_UNREACHABLE через reader-сервис, сброс соединения через прокси, 04.10.2026); данные не изменены</t>
-        </is>
-      </c>
-      <c r="AH11" s="4" t="inlineStr">
+• Перепроверка: Сайт ambou.edu.et недоступен (ERR_ADDRESS_UNREACHABLE через reader-сервис, сброс соединения через прокси, 04.10.2026); данные не изменены
+• Ручная проверка: Рейтинги: QS 2027 — официальный файл данных topuniversities.com (qs-rankings-data/en/4153156.txt), сверка 05.10.2026; THE 2027 — список THE World University Rankings 2027 (data/sources/the2027.json). Webometrics: webometrics.info не открывается (DNS) — не заполнено</t>
+        </is>
+      </c>
+      <c r="AI11" s="4" t="inlineStr">
         <is>
           <t>• Https://www.ambou.edu.et (HTTP 500 database error, Oct 2026)
 • Https://t.me/s/AmboUniversityOfficial</t>
         </is>
       </c>
-      <c r="AI11" s="4" t="inlineStr">
+      <c r="AJ11" s="4" t="inlineStr">
         <is>
           <t>2026-10-05</t>
         </is>
       </c>
-      <c r="AJ11" s="4" t="inlineStr"/>
+      <c r="AK11" s="4" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
@@ -3202,60 +3438,79 @@
           <t>President</t>
         </is>
       </c>
-      <c r="S12" s="4" t="inlineStr"/>
-      <c r="T12" s="4" t="inlineStr"/>
-      <c r="U12" s="4" t="inlineStr"/>
-      <c r="V12" s="4" t="n">
+      <c r="S12" s="4" t="inlineStr">
+        <is>
+          <t>QS2027: не в рейтинге</t>
+        </is>
+      </c>
+      <c r="T12" s="4" t="inlineStr">
+        <is>
+          <t>THE2027: не в рейтинге</t>
+        </is>
+      </c>
+      <c r="U12" s="4" t="inlineStr">
+        <is>
+          <t>нет общенационального рейтинга</t>
+        </is>
+      </c>
+      <c r="V12" s="4" t="inlineStr">
+        <is>
+          <t>3299</t>
+        </is>
+      </c>
+      <c r="W12" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="W12" s="4" t="inlineStr"/>
       <c r="X12" s="4" t="inlineStr"/>
       <c r="Y12" s="4" t="inlineStr"/>
       <c r="Z12" s="4" t="inlineStr"/>
       <c r="AA12" s="4" t="inlineStr"/>
       <c r="AB12" s="4" t="inlineStr"/>
-      <c r="AC12" s="4" t="n">
+      <c r="AC12" s="4" t="inlineStr"/>
+      <c r="AD12" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="AD12" s="8" t="inlineStr">
+      <c r="AE12" s="8" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="AE12" s="4" t="inlineStr">
+      <c r="AF12" s="4" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="AF12" s="4" t="inlineStr">
+      <c r="AG12" s="4" t="inlineStr">
         <is>
           <t>средняя</t>
         </is>
       </c>
-      <c r="AG12" s="4" t="inlineStr">
+      <c r="AH12" s="4" t="inlineStr">
         <is>
           <t>• Спутников на орбите не найдено (проверка: nanosats.csv и поиск 'Ethiopian university CubeSat launched', окт. 2026)
 • Президент Dr.-Ing. Abdella Kemal подтверждён новостями сайта от 25–28.09.2026
 • Profile_type 'technical/aerospace' условно — ядро университета инженерно-водохозяйственное (AWTI, AMiT); аэрокосмических подразделений не найдено
 • Corcom@amu.edu.et — адрес службы корпоративных коммуникаций (общий адрес сайта); e-mail Директората интернационализации и сотрудничества не опубликован; партнёрствами также занимается офис GCPM при вице-президенте по исследованиям
-• Тел. +251 46 881 0771 — офис президента (Management Building); пресс-служба: +251 46 881 4986</t>
-        </is>
-      </c>
-      <c r="AH12" s="4" t="inlineStr">
+• Тел. +251 46 881 0771 — офис президента (Management Building); пресс-служба: +251 46 881 4986
+• Рейтинги: Национального рейтинга с местами нет: МинОбр Эфиопии делит гос. вузы на категории (research / applied science / general), мест не публикует</t>
+        </is>
+      </c>
+      <c r="AI12" s="4" t="inlineStr">
         <is>
           <t>• Https://www.amu.edu.et/en/
 • Https://www.amu.edu.et/en/administration/presidents-office/amu-president
 • Https://www.amu.edu.et/en/amu-holds-annual-grants-and-publication-day-honors-excellence-in-research-grant-acquisition-and-scholarly-publication
 • Https://www.amu.edu.et/en/amu-sifa-project-undergoes-progress-monitoring-with-donors-and-stakeholders
-• Https://www.amu.edu.et/en/partnership/our-partners/international-partners</t>
-        </is>
-      </c>
-      <c r="AI12" s="4" t="inlineStr">
+• Https://www.amu.edu.et/en/partnership/our-partners/international-partners
+https://figshare.com/articles/preprint/Ranking_Web_of_Universities_webometrics_info_July_2026_edition/33062150</t>
+        </is>
+      </c>
+      <c r="AJ12" s="4" t="inlineStr">
         <is>
           <t>2026-10-05</t>
         </is>
       </c>
-      <c r="AJ12" s="4" t="inlineStr"/>
+      <c r="AK12" s="4" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
@@ -3353,44 +3608,62 @@
           <t>President</t>
         </is>
       </c>
-      <c r="S13" s="4" t="inlineStr"/>
-      <c r="T13" s="4" t="inlineStr"/>
-      <c r="U13" s="4" t="inlineStr"/>
-      <c r="V13" s="4" t="n">
+      <c r="S13" s="4" t="inlineStr">
+        <is>
+          <t>QS2027: не в рейтинге</t>
+        </is>
+      </c>
+      <c r="T13" s="4" t="inlineStr">
+        <is>
+          <t>THE2027: не в рейтинге</t>
+        </is>
+      </c>
+      <c r="U13" s="4" t="inlineStr">
+        <is>
+          <t>нет общенационального рейтинга</t>
+        </is>
+      </c>
+      <c r="V13" s="4" t="inlineStr">
+        <is>
+          <t>нет в опубл. списке</t>
+        </is>
+      </c>
+      <c r="W13" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="W13" s="4" t="inlineStr"/>
       <c r="X13" s="4" t="inlineStr"/>
       <c r="Y13" s="4" t="inlineStr"/>
       <c r="Z13" s="4" t="inlineStr"/>
       <c r="AA13" s="4" t="inlineStr"/>
       <c r="AB13" s="4" t="inlineStr"/>
-      <c r="AC13" s="4" t="n">
+      <c r="AC13" s="4" t="inlineStr"/>
+      <c r="AD13" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="AD13" s="8" t="inlineStr">
+      <c r="AE13" s="8" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="AE13" s="4" t="inlineStr">
+      <c r="AF13" s="4" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="AF13" s="4" t="inlineStr">
+      <c r="AG13" s="4" t="inlineStr">
         <is>
           <t>средняя</t>
         </is>
       </c>
-      <c r="AG13" s="4" t="inlineStr">
+      <c r="AH13" s="4" t="inlineStr">
         <is>
           <t>• Единственный опубликованный институциональный ящик — pir@asu.edu.et (Public and International Relations Executive, тел. +251 57 887 5057); имя руководителя офиса на сайте не указано
 • Президент Dr. Yared Mulu (на сайте личный gmail yaredmulugelaw@gmail.com, тел. +251 577 750 977)
-• Регион Бенишангуль-Гумуз (рядом плотина GERD); спутниковых проектов не найдено</t>
-        </is>
-      </c>
-      <c r="AH13" s="4" t="inlineStr">
+• Регион Бенишангуль-Гумуз (рядом плотина GERD); спутниковых проектов не найдено
+• Рейтинги: Национального рейтинга с местами нет: МинОбр Эфиопии делит гос. вузы на категории (research / applied science / general), мест не публикует</t>
+        </is>
+      </c>
+      <c r="AI13" s="4" t="inlineStr">
         <is>
           <t>• Https://asu.edu.et
 • Https://asu.edu.et (Message from the President
@@ -3401,12 +3674,12 @@
 • Nanosats.csv (nation=Ethiopia: only ESSTI ET-SMART-RSS and cancelled AAiT ET-SAT)</t>
         </is>
       </c>
-      <c r="AI13" s="4" t="inlineStr">
+      <c r="AJ13" s="4" t="inlineStr">
         <is>
           <t>2026-10-05</t>
         </is>
       </c>
-      <c r="AJ13" s="4" t="inlineStr"/>
+      <c r="AK13" s="4" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
@@ -3505,44 +3778,62 @@
           <t>President</t>
         </is>
       </c>
-      <c r="S14" s="4" t="inlineStr"/>
-      <c r="T14" s="4" t="inlineStr"/>
-      <c r="U14" s="4" t="inlineStr"/>
-      <c r="V14" s="4" t="n">
+      <c r="S14" s="4" t="inlineStr">
+        <is>
+          <t>QS2027: не в рейтинге</t>
+        </is>
+      </c>
+      <c r="T14" s="4" t="inlineStr">
+        <is>
+          <t>THE2027: не в рейтинге</t>
+        </is>
+      </c>
+      <c r="U14" s="4" t="inlineStr">
+        <is>
+          <t>нет общенационального рейтинга</t>
+        </is>
+      </c>
+      <c r="V14" s="4" t="inlineStr">
+        <is>
+          <t>нет в опубл. списке</t>
+        </is>
+      </c>
+      <c r="W14" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="W14" s="4" t="inlineStr"/>
       <c r="X14" s="4" t="inlineStr"/>
       <c r="Y14" s="4" t="inlineStr"/>
       <c r="Z14" s="4" t="inlineStr"/>
       <c r="AA14" s="4" t="inlineStr"/>
       <c r="AB14" s="4" t="inlineStr"/>
-      <c r="AC14" s="4" t="n">
+      <c r="AC14" s="4" t="inlineStr"/>
+      <c r="AD14" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="AD14" s="8" t="inlineStr">
+      <c r="AE14" s="8" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="AE14" s="4" t="inlineStr">
+      <c r="AF14" s="4" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="AF14" s="4" t="inlineStr">
+      <c r="AG14" s="4" t="inlineStr">
         <is>
           <t>средняя</t>
         </is>
       </c>
-      <c r="AG14" s="4" t="inlineStr">
+      <c r="AH14" s="4" t="inlineStr">
         <is>
           <t>• Research, International Relations and Partnership Directorate (RIRPD) создан в конце декабря (по сайту); директор Anteneh Fikrie (Asst. Prof.), также anteneh.fikrie@bhu.edu.et, тел. +251 922 46 51 29
 • Президент публикует личный рабочий e-mail temesgendebelo@bhu.edu.et — можно поставить в копию
-• Регион Западный Гуджи (Оромия) — возможны проблемы с безопасностью; спутниковых проектов не найдено</t>
-        </is>
-      </c>
-      <c r="AH14" s="4" t="inlineStr">
+• Регион Западный Гуджи (Оромия) — возможны проблемы с безопасностью; спутниковых проектов не найдено
+• Рейтинги: Национального рейтинга с местами нет: МинОбр Эфиопии делит гос. вузы на категории (research / applied science / general), мест не публикует</t>
+        </is>
+      </c>
+      <c r="AI14" s="4" t="inlineStr">
         <is>
           <t>• Https://www.bhu.edu.et
 • Https://www.bhu.edu.et (President's Message)
@@ -3552,12 +3843,12 @@
 • Nanosats.csv (nation=Ethiopia: only ESSTI ET-SMART-RSS and cancelled AAiT ET-SAT)</t>
         </is>
       </c>
-      <c r="AI14" s="4" t="inlineStr">
+      <c r="AJ14" s="4" t="inlineStr">
         <is>
           <t>2026-10-05</t>
         </is>
       </c>
-      <c r="AJ14" s="4" t="inlineStr"/>
+      <c r="AK14" s="4" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
@@ -3656,58 +3947,77 @@
           <t>President</t>
         </is>
       </c>
-      <c r="S15" s="4" t="inlineStr"/>
-      <c r="T15" s="4" t="inlineStr"/>
-      <c r="U15" s="4" t="inlineStr"/>
-      <c r="V15" s="4" t="n">
+      <c r="S15" s="4" t="inlineStr">
+        <is>
+          <t>QS2027: не в рейтинге</t>
+        </is>
+      </c>
+      <c r="T15" s="4" t="inlineStr">
+        <is>
+          <t>THE2027: не в рейтинге</t>
+        </is>
+      </c>
+      <c r="U15" s="4" t="inlineStr">
+        <is>
+          <t>нет общенационального рейтинга</t>
+        </is>
+      </c>
+      <c r="V15" s="4" t="inlineStr">
+        <is>
+          <t>4631</t>
+        </is>
+      </c>
+      <c r="W15" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="W15" s="4" t="inlineStr"/>
       <c r="X15" s="4" t="inlineStr"/>
       <c r="Y15" s="4" t="inlineStr"/>
       <c r="Z15" s="4" t="inlineStr"/>
       <c r="AA15" s="4" t="inlineStr"/>
       <c r="AB15" s="4" t="inlineStr"/>
-      <c r="AC15" s="4" t="n">
+      <c r="AC15" s="4" t="inlineStr"/>
+      <c r="AD15" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="AD15" s="8" t="inlineStr">
+      <c r="AE15" s="8" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="AE15" s="4" t="inlineStr">
+      <c r="AF15" s="4" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="AF15" s="4" t="inlineStr">
+      <c r="AG15" s="4" t="inlineStr">
         <is>
           <t>средняя</t>
         </is>
       </c>
-      <c r="AG15" s="4" t="inlineStr">
+      <c r="AH15" s="4" t="inlineStr">
         <is>
           <t>• Международный отдел: International Relation and Partnership Director — Dr. Bethel Geremew Shefine (bethel@dbu.edu.et, моб. +251 919 396 017); дата страницы контактов не указана — актуальность на 2026 не подтверждена
 • Dbu@dbu.edu.et — ящик Executive Office of Public and International Relations (исполнительный директор Genzeb Atalay Nigatu, Asst. Prof.)
-• С 2020 г. — University of Applied Sciences; регион Амхара (возможны проблемы с безопасностью); спутниковых проектов не найдено</t>
-        </is>
-      </c>
-      <c r="AH15" s="4" t="inlineStr">
+• С 2020 г. — University of Applied Sciences; регион Амхара (возможны проблемы с безопасностью); спутниковых проектов не найдено
+• Рейтинги: Национального рейтинга с местами нет: МинОбр Эфиопии делит гос. вузы на категории (research / applied science / general), мест не публикует</t>
+        </is>
+      </c>
+      <c r="AI15" s="4" t="inlineStr">
         <is>
           <t>• Https://www.dbu.edu.et
 • Https://www.dbu.edu.et/dbu_contact
 • Https://www.dbu.edu.et/president_message
 • Https://www.wearetech.africa/en/fils-uk/news/tech/ethiopia-expands-space-program-with-2026-satellite-launch (general check: no Ethiopian university-built satellite)
-• Nanosats.csv (nation=Ethiopia: only ESSTI ET-SMART-RSS and cancelled AAiT ET-SAT)</t>
-        </is>
-      </c>
-      <c r="AI15" s="4" t="inlineStr">
+• Nanosats.csv (nation=Ethiopia: only ESSTI ET-SMART-RSS and cancelled AAiT ET-SAT)
+https://figshare.com/articles/preprint/Ranking_Web_of_Universities_webometrics_info_July_2026_edition/33062150</t>
+        </is>
+      </c>
+      <c r="AJ15" s="4" t="inlineStr">
         <is>
           <t>2026-10-05</t>
         </is>
       </c>
-      <c r="AJ15" s="4" t="inlineStr"/>
+      <c r="AK15" s="4" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">
@@ -3806,58 +4116,77 @@
           <t>President</t>
         </is>
       </c>
-      <c r="S16" s="4" t="inlineStr"/>
-      <c r="T16" s="4" t="inlineStr"/>
-      <c r="U16" s="4" t="inlineStr"/>
-      <c r="V16" s="4" t="n">
+      <c r="S16" s="4" t="inlineStr">
+        <is>
+          <t>QS2027: не в рейтинге</t>
+        </is>
+      </c>
+      <c r="T16" s="4" t="inlineStr">
+        <is>
+          <t>THE2027: не в рейтинге</t>
+        </is>
+      </c>
+      <c r="U16" s="4" t="inlineStr">
+        <is>
+          <t>нет общенационального рейтинга</t>
+        </is>
+      </c>
+      <c r="V16" s="4" t="inlineStr">
+        <is>
+          <t>4866</t>
+        </is>
+      </c>
+      <c r="W16" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="W16" s="4" t="inlineStr"/>
       <c r="X16" s="4" t="inlineStr"/>
       <c r="Y16" s="4" t="inlineStr"/>
       <c r="Z16" s="4" t="inlineStr"/>
       <c r="AA16" s="4" t="inlineStr"/>
       <c r="AB16" s="4" t="inlineStr"/>
-      <c r="AC16" s="4" t="n">
+      <c r="AC16" s="4" t="inlineStr"/>
+      <c r="AD16" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="AD16" s="8" t="inlineStr">
+      <c r="AE16" s="8" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="AE16" s="4" t="inlineStr">
+      <c r="AF16" s="4" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="AF16" s="4" t="inlineStr">
+      <c r="AG16" s="4" t="inlineStr">
         <is>
           <t>средняя</t>
         </is>
       </c>
-      <c r="AG16" s="4" t="inlineStr">
+      <c r="AH16" s="4" t="inlineStr">
         <is>
           <t>• Спутников на орбите не найдено (проверка: nanosats.csv и поиск 'Ethiopian university CubeSat launched', окт. 2026)
 • Президент Dr. Sayeh Kassaw назначен Минобразования 24.01.2024 (шестой президент); личный e-mail: Sayeh_kassaw@dmu.edu.et, тел. +251 58 771 1646
 • Директорат международных связей в исследованиях и партнёрствах: директор Getnet Atenafu (PhD, доцент), тел. +251 912 080 282, личный gmail getnet.atenafu@gmail.com; официальный ящик директората — projectd.partnership@dmu.edu.et
-• Prcd@dmu.edu.et — общий адрес в шапке сайта (по-видимому, директорат по связям с общественностью)</t>
-        </is>
-      </c>
-      <c r="AH16" s="4" t="inlineStr">
+• Prcd@dmu.edu.et — общий адрес в шапке сайта (по-видимому, директорат по связям с общественностью)
+• Рейтинги: Национального рейтинга с местами нет: МинОбр Эфиопии делит гос. вузы на категории (research / applied science / general), мест не публикует</t>
+        </is>
+      </c>
+      <c r="AI16" s="4" t="inlineStr">
         <is>
           <t>• Https://www.dmu.edu.et/
 • Https://www.dmu.edu.et/?page_id=469
 • Https://www.dmu.edu.et/?page_id=1349
-• Https://www.dmu.edu.et/?page_id=562</t>
-        </is>
-      </c>
-      <c r="AI16" s="4" t="inlineStr">
+• Https://www.dmu.edu.et/?page_id=562
+https://figshare.com/articles/preprint/Ranking_Web_of_Universities_webometrics_info_July_2026_edition/33062150</t>
+        </is>
+      </c>
+      <c r="AJ16" s="4" t="inlineStr">
         <is>
           <t>2026-10-05</t>
         </is>
       </c>
-      <c r="AJ16" s="4" t="inlineStr"/>
+      <c r="AK16" s="4" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="4" t="n">
@@ -3948,58 +4277,68 @@
           <t>President</t>
         </is>
       </c>
-      <c r="S17" s="4" t="inlineStr"/>
-      <c r="T17" s="4" t="inlineStr"/>
+      <c r="S17" s="4" t="inlineStr">
+        <is>
+          <t>QS2027: не в рейтинге</t>
+        </is>
+      </c>
+      <c r="T17" s="4" t="inlineStr">
+        <is>
+          <t>THE2027: не в рейтинге</t>
+        </is>
+      </c>
       <c r="U17" s="4" t="inlineStr"/>
-      <c r="V17" s="4" t="n">
+      <c r="V17" s="4" t="inlineStr"/>
+      <c r="W17" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="W17" s="4" t="inlineStr"/>
       <c r="X17" s="4" t="inlineStr"/>
       <c r="Y17" s="4" t="inlineStr"/>
       <c r="Z17" s="4" t="inlineStr"/>
       <c r="AA17" s="4" t="inlineStr"/>
       <c r="AB17" s="4" t="inlineStr"/>
-      <c r="AC17" s="4" t="n">
+      <c r="AC17" s="4" t="inlineStr"/>
+      <c r="AD17" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="AD17" s="8" t="inlineStr">
+      <c r="AE17" s="8" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="AE17" s="4" t="inlineStr">
+      <c r="AF17" s="4" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="AF17" s="4" t="inlineStr">
+      <c r="AG17" s="4" t="inlineStr">
         <is>
           <t>средняя</t>
         </is>
       </c>
-      <c r="AG17" s="4" t="inlineStr">
+      <c r="AH17" s="4" t="inlineStr">
         <is>
           <t>• Спутников на орбите не найдено (проверка: nanosats.csv и поиск 'Ethiopian university CubeSat launched', окт. 2026)
 • Сайт dtu.edu.et блокирует наши запросы (редирект на страницу блокировки) — данные взяты из официального Telegram-канала университета
 • Президент Dr. Solomon Abegaze упомянут как президент в посте от 25.09.2026; в марте 2025 СМИ называли президентом Anegagregn Gashaw — смена руководства
 • Сентябрь 2026: идёт конкурс на должности вице-президентов
 • Телефон, почтовый ящик и e-mail международного отдела не подтверждены; dtu@dtu.edu.et — официальный общий адрес, указанный в Telegram-канале
-• Перепроверка: 04.10.2026: сайт dtu.edu.et по-прежнему блокирует доступ; президент Dr. Solomon Abegaze повторно подтверждён в последних постах официального Telegram-канала (сентябрь 2026); телефон и международный e-mail не найдены</t>
-        </is>
-      </c>
-      <c r="AH17" s="4" t="inlineStr">
+• Перепроверка: 04.10.2026: сайт dtu.edu.et по-прежнему блокирует доступ; президент Dr. Solomon Abegaze повторно подтверждён в последних постах официального Telegram-канала (сентябрь 2026); телефон и международный e-mail не найдены
+• Ручная проверка: Рейтинги: QS 2027 — официальный файл данных topuniversities.com (qs-rankings-data/en/4153156.txt), сверка 05.10.2026; THE 2027 — список THE World University Rankings 2027 (data/sources/the2027.json). Webometrics: webometrics.info не открывается (DNS) — не заполнено</t>
+        </is>
+      </c>
+      <c r="AI17" s="4" t="inlineStr">
         <is>
           <t>• Https://t.me/s/DTUniversity (official DTU Telegram channel, posts Sep 2026)
 • Https://dtu.edu.et (blocked from our network)</t>
         </is>
       </c>
-      <c r="AI17" s="4" t="inlineStr">
+      <c r="AJ17" s="4" t="inlineStr">
         <is>
           <t>2026-10-05</t>
         </is>
       </c>
-      <c r="AJ17" s="4" t="inlineStr"/>
+      <c r="AK17" s="4" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="4" t="n">
@@ -4098,44 +4437,62 @@
           <t>President</t>
         </is>
       </c>
-      <c r="S18" s="4" t="inlineStr"/>
-      <c r="T18" s="4" t="inlineStr"/>
-      <c r="U18" s="4" t="inlineStr"/>
-      <c r="V18" s="4" t="n">
+      <c r="S18" s="4" t="inlineStr">
+        <is>
+          <t>QS2027: не в рейтинге</t>
+        </is>
+      </c>
+      <c r="T18" s="4" t="inlineStr">
+        <is>
+          <t>THE2027: не в рейтинге</t>
+        </is>
+      </c>
+      <c r="U18" s="4" t="inlineStr">
+        <is>
+          <t>нет общенационального рейтинга</t>
+        </is>
+      </c>
+      <c r="V18" s="4" t="inlineStr">
+        <is>
+          <t>нет в опубл. списке</t>
+        </is>
+      </c>
+      <c r="W18" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="W18" s="4" t="inlineStr"/>
       <c r="X18" s="4" t="inlineStr"/>
       <c r="Y18" s="4" t="inlineStr"/>
       <c r="Z18" s="4" t="inlineStr"/>
       <c r="AA18" s="4" t="inlineStr"/>
       <c r="AB18" s="4" t="inlineStr"/>
-      <c r="AC18" s="4" t="n">
+      <c r="AC18" s="4" t="inlineStr"/>
+      <c r="AD18" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="AD18" s="8" t="inlineStr">
+      <c r="AE18" s="8" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="AE18" s="4" t="inlineStr">
+      <c r="AF18" s="4" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="AF18" s="4" t="inlineStr">
+      <c r="AG18" s="4" t="inlineStr">
         <is>
           <t>средняя</t>
         </is>
       </c>
-      <c r="AG18" s="4" t="inlineStr">
+      <c r="AH18" s="4" t="inlineStr">
         <is>
           <t>• Адрес президента опубликован как 'presidant@du.edu.et' (так на сайте, возможна опечатка — при недоставке использовать pirdir@du.edu.et)
 • Public &amp; International Relations: директор Habtamu Mesfin; на странице контактов у него указан drdir@du.edu.et, а в шапке сайта — pirdir@du.edu.et (выбран pirdir@ как основной ящик офиса)
-• Страницы Internationalization &amp; Partnership и списка президентов пустые; спутниковых проектов не найдено</t>
-        </is>
-      </c>
-      <c r="AH18" s="4" t="inlineStr">
+• Страницы Internationalization &amp; Partnership и списка президентов пустые; спутниковых проектов не найдено
+• Рейтинги: Национального рейтинга с местами нет: МинОбр Эфиопии делит гос. вузы на категории (research / applied science / general), мест не публикует</t>
+        </is>
+      </c>
+      <c r="AI18" s="4" t="inlineStr">
         <is>
           <t>• Https://www.du.edu.et
 • Https://www.du.edu.et/contact/
@@ -4144,12 +4501,12 @@
 • Nanosats.csv (nation=Ethiopia: only ESSTI ET-SMART-RSS and cancelled AAiT ET-SAT)</t>
         </is>
       </c>
-      <c r="AI18" s="4" t="inlineStr">
+      <c r="AJ18" s="4" t="inlineStr">
         <is>
           <t>2026-10-05</t>
         </is>
       </c>
-      <c r="AJ18" s="4" t="inlineStr"/>
+      <c r="AK18" s="4" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="4" t="n">
@@ -4240,44 +4597,62 @@
           <t>President</t>
         </is>
       </c>
-      <c r="S19" s="4" t="inlineStr"/>
-      <c r="T19" s="4" t="inlineStr"/>
-      <c r="U19" s="4" t="inlineStr"/>
-      <c r="V19" s="4" t="n">
+      <c r="S19" s="4" t="inlineStr">
+        <is>
+          <t>QS2027: не в рейтинге</t>
+        </is>
+      </c>
+      <c r="T19" s="4" t="inlineStr">
+        <is>
+          <t>THE2027: не в рейтинге</t>
+        </is>
+      </c>
+      <c r="U19" s="4" t="inlineStr">
+        <is>
+          <t>нет общенационального рейтинга</t>
+        </is>
+      </c>
+      <c r="V19" s="4" t="inlineStr">
+        <is>
+          <t>нет в опубл. списке</t>
+        </is>
+      </c>
+      <c r="W19" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="W19" s="4" t="inlineStr"/>
       <c r="X19" s="4" t="inlineStr"/>
       <c r="Y19" s="4" t="inlineStr"/>
       <c r="Z19" s="4" t="inlineStr"/>
       <c r="AA19" s="4" t="inlineStr"/>
       <c r="AB19" s="4" t="inlineStr"/>
-      <c r="AC19" s="4" t="n">
+      <c r="AC19" s="4" t="inlineStr"/>
+      <c r="AD19" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="AD19" s="8" t="inlineStr">
+      <c r="AE19" s="8" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="AE19" s="4" t="inlineStr">
+      <c r="AF19" s="4" t="inlineStr">
         <is>
           <t>нет</t>
         </is>
       </c>
-      <c r="AF19" s="4" t="inlineStr">
+      <c r="AG19" s="4" t="inlineStr">
         <is>
           <t>средняя</t>
         </is>
       </c>
-      <c r="AG19" s="4" t="inlineStr">
+      <c r="AH19" s="4" t="inlineStr">
         <is>
           <t>• Общий e-mail, телефон и P.O. Box на сайте не опубликованы (на странице контактов заглушки)
 • Office of International Partnerships: директор Dawit Daniel (Asst. Prof.), личный адрес dawit.daniel@ddu.edu.et; отдельно есть International and Public Relations Directorate — директор Tensay Hailu (Asst. Prof.)
-• Университет переходит в статус University of Applied Sciences; спутниковых проектов не найдено</t>
-        </is>
-      </c>
-      <c r="AH19" s="4" t="inlineStr">
+• Университет переходит в статус University of Applied Sciences; спутниковых проектов не найдено
+• Рейтинги: Национального рейтинга с местами нет: МинОбр Эфиопии делит гос. вузы на категории (research / applied science / general), мест не публикует</t>
+        </is>
+      </c>
+      <c r="AI19" s="4" t="inlineStr">
         <is>
           <t>• Https://www.ddu.edu.et
 • Https://www.ddu.edu.et/presidents-3/
@@ -4288,12 +4663,12 @@
 • Nanosats.csv (nation=Ethiopia: only ESSTI ET-SMART-RSS and cancelled AAiT ET-SAT)</t>
         </is>
       </c>
-      <c r="AI19" s="4" t="inlineStr">
+      <c r="AJ19" s="4" t="inlineStr">
         <is>
           <t>2026-10-05</t>
         </is>
       </c>
-      <c r="AJ19" s="4" t="inlineStr"/>
+      <c r="AK19" s="4" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="4" t="n">
@@ -4365,41 +4740,51 @@
           <t>President</t>
         </is>
       </c>
-      <c r="S20" s="4" t="inlineStr"/>
-      <c r="T20" s="4" t="inlineStr"/>
+      <c r="S20" s="4" t="inlineStr">
+        <is>
+          <t>QS2027: не в рейтинге</t>
+        </is>
+      </c>
+      <c r="T20" s="4" t="inlineStr">
+        <is>
+          <t>THE2027: не в рейтинге</t>
+        </is>
+      </c>
       <c r="U20" s="4" t="inlineStr"/>
-      <c r="V20" s="4" t="n">
+      <c r="V20" s="4" t="inlineStr"/>
+      <c r="W20" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="W20" s="4" t="inlineStr"/>
       <c r="X20" s="4" t="inlineStr"/>
       <c r="Y20" s="4" t="inlineStr"/>
       <c r="Z20" s="4" t="inlineStr"/>
       <c r="AA20" s="4" t="inlineStr"/>
       <c r="AB20" s="4" t="inlineStr"/>
-      <c r="AC20" s="4" t="n">
+      <c r="AC20" s="4" t="inlineStr"/>
+      <c r="AD20" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="AD20" s="8" t="inlineStr">
+      <c r="AE20" s="8" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="AE20" s="4" t="inlineStr"/>
-      <c r="AF20" s="4" t="inlineStr">
+      <c r="AF20" s="4" t="inlineStr"/>
+      <c r="AG20" s="4" t="inlineStr">
         <is>
           <t>низкая</t>
         </is>
       </c>
-      <c r="AG20" s="4" t="inlineStr">
+      <c r="AH20" s="4" t="inlineStr">
         <is>
           <t>• Официальный сайт ecsu.edu.et недоступен (сброс соединения / 503) — контакты и руководство не проверены, нужна ручная проверка
 • В Википедии упоминается также домен epsu.edu.et (возможно, переименование в Ethiopian Public Service University) и президент Nigus Tadese (PhD) — не подтверждено на 2026; домен epsu.edu.et тоже недоступен
 • Вуз государственной службы (управление, политика, право) — низкая релевантность для спутниковой программы; спутниковых проектов не найдено
-• Перепроверка: Сайты ecsu.edu.et / epsu.edu.et по-прежнему недоступны (04.10.2026); в списке университетов на moe.gov.et вуз не значится; данные не изменены</t>
-        </is>
-      </c>
-      <c r="AH20" s="4" t="inlineStr">
+• Перепроверка: Сайты ecsu.edu.et / epsu.edu.et по-прежнему недоступны (04.10.2026); в списке университетов на moe.gov.et вуз не значится; данные не изменены
+• Ручная проверка: Рейтинги: QS 2027 — официальный файл данных topuniversities.com (qs-rankings-data/en/4153156.txt), сверка 05.10.2026; THE 2027 — список THE World University Rankings 2027 (data/sources/the2027.json). Webometrics: webometrics.info не открывается (DNS) — не заполнено</t>
+        </is>
+      </c>
+      <c r="AI20" s="4" t="inlineStr">
         <is>
           <t>• Https://www.ecsu.edu.et (unreachable: connection reset / HTTP 503, Oct 2026)
 • Https://en.wikipedia.org/wiki/Ethiopian_Civil_Service_University
@@ -4407,12 +4792,12 @@
 • Nanosats.csv (nation=Ethiopia: only ESSTI ET-SMART-RSS and cancelled AAiT ET-SAT)</t>
         </is>
       </c>
-      <c r="AI20" s="4" t="inlineStr">
+      <c r="AJ20" s="4" t="inlineStr">
         <is>
           <t>2026-10-05</t>
         </is>
       </c>
-      <c r="AJ20" s="4" t="inlineStr"/>
+      <c r="AK20" s="4" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="4" t="n">
@@ -4488,33 +4873,42 @@
           <t>President</t>
         </is>
       </c>
-      <c r="S21" s="4" t="inlineStr"/>
-      <c r="T21" s="4" t="inlineStr"/>
+      <c r="S21" s="4" t="inlineStr">
+        <is>
+          <t>QS2027: не в рейтинге</t>
+        </is>
+      </c>
+      <c r="T21" s="4" t="inlineStr">
+        <is>
+          <t>THE2027: не в рейтинге</t>
+        </is>
+      </c>
       <c r="U21" s="4" t="inlineStr"/>
-      <c r="V21" s="4" t="n">
+      <c r="V21" s="4" t="inlineStr"/>
+      <c r="W21" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="W21" s="4" t="inlineStr"/>
       <c r="X21" s="4" t="inlineStr"/>
       <c r="Y21" s="4" t="inlineStr"/>
       <c r="Z21" s="4" t="inlineStr"/>
       <c r="AA21" s="4" t="inlineStr"/>
       <c r="AB21" s="4" t="inlineStr"/>
-      <c r="AC21" s="4" t="n">
+      <c r="AC21" s="4" t="inlineStr"/>
+      <c r="AD21" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="AD21" s="8" t="inlineStr">
+      <c r="AE21" s="8" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="AE21" s="4" t="inlineStr"/>
-      <c r="AF21" s="4" t="inlineStr">
+      <c r="AF21" s="4" t="inlineStr"/>
+      <c r="AG21" s="4" t="inlineStr">
         <is>
           <t>низкая</t>
         </is>
       </c>
-      <c r="AG21" s="4" t="inlineStr">
+      <c r="AH21" s="4" t="inlineStr">
         <is>
           <t>• Спутников на орбите не найдено (проверка: nanosats.csv и поиск 'Ethiopian university CubeSat launched', окт. 2026)
 • Президент Dr. Diriba Eticha Tujuba (PhD) указан на главной странице; новость от 09.04.2026 упоминает его как президента (Dr. Diriba Iticha)
@@ -4522,22 +4916,23 @@
 • По поисковой выдаче (старая версия сайта, не открылась): info@gmu.edu.et, тел. +251 47 551 1923 — НЕ подтверждено, в поля не внесено
 • Существует Директорат исследований, международных связей и партнёрств, но его руководитель и e-mail не опубликованы
 • Повторная проверка 04.10.2026: главная страница gmu.edu.et (©2026) по-прежнему называет президентом Dr. Diriba Eticha Tujuba; страницы President Office и Contact Us рендерятся JS без контактов — e-mail/телефон не подтверждены
-• Перепроверка: Президент повторно подтверждён на сайте (новости 2026), но официальных e-mail/телефона нет — уровень low сохранён</t>
-        </is>
-      </c>
-      <c r="AH21" s="4" t="inlineStr">
+• Перепроверка: Президент повторно подтверждён на сайте (новости 2026), но официальных e-mail/телефона нет — уровень low сохранён
+• Ручная проверка: Рейтинги: QS 2027 — официальный файл данных topuniversities.com (qs-rankings-data/en/4153156.txt), сверка 05.10.2026; THE 2027 — список THE World University Rankings 2027 (data/sources/the2027.json). Webometrics: webometrics.info не открывается (DNS) — не заполнено</t>
+        </is>
+      </c>
+      <c r="AI21" s="4" t="inlineStr">
         <is>
           <t>• Https://www.gmu.edu.et/
 • Https://www.gmu.edu.et/administration/president-office1
 • Https://www.gmu.edu.et/contact-us</t>
         </is>
       </c>
-      <c r="AI21" s="4" t="inlineStr">
+      <c r="AJ21" s="4" t="inlineStr">
         <is>
           <t>2026-10-05</t>
         </is>
       </c>
-      <c r="AJ21" s="4" t="inlineStr"/>
+      <c r="AK21" s="4" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="4" t="n">
@@ -4631,45 +5026,63 @@
           <t>President</t>
         </is>
       </c>
-      <c r="S22" s="4" t="inlineStr"/>
-      <c r="T22" s="4" t="inlineStr"/>
-      <c r="U22" s="4" t="inlineStr"/>
-      <c r="V22" s="4" t="n">
+      <c r="S22" s="4" t="inlineStr">
+        <is>
+          <t>QS2027: не в рейтинге</t>
+        </is>
+      </c>
+      <c r="T22" s="4" t="inlineStr">
+        <is>
+          <t>THE2027: не в рейтинге</t>
+        </is>
+      </c>
+      <c r="U22" s="4" t="inlineStr">
+        <is>
+          <t>нет общенационального рейтинга</t>
+        </is>
+      </c>
+      <c r="V22" s="4" t="inlineStr">
+        <is>
+          <t>3035</t>
+        </is>
+      </c>
+      <c r="W22" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="W22" s="4" t="inlineStr"/>
       <c r="X22" s="4" t="inlineStr"/>
       <c r="Y22" s="4" t="inlineStr"/>
       <c r="Z22" s="4" t="inlineStr"/>
       <c r="AA22" s="4" t="inlineStr"/>
       <c r="AB22" s="4" t="inlineStr"/>
-      <c r="AC22" s="4" t="n">
+      <c r="AC22" s="4" t="inlineStr"/>
+      <c r="AD22" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="AD22" s="8" t="inlineStr">
+      <c r="AE22" s="8" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="AE22" s="4" t="inlineStr">
+      <c r="AF22" s="4" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="AF22" s="4" t="inlineStr">
+      <c r="AG22" s="4" t="inlineStr">
         <is>
           <t>высокая</t>
         </is>
       </c>
-      <c r="AG22" s="4" t="inlineStr">
+      <c r="AH22" s="4" t="inlineStr">
         <is>
           <t>• Президент с 27.12.2019 Dr. Jemal Yousuf Hassen; подтверждён в новости 2026 (QS Africa Forum 2026); личный e-mail на сайте — yahoo (jemaly2001@yahoo.com), тел. офиса +251 25 553 0319
 • Официального ящика международного отдела нет; Public and International Relations Directorate — директор Mr. Alemishet (Alemeshet) Teshome, только личный yahoo (sportalem@yahoo.com) — поэтому письмо на общий адрес haramaya@haramaya.edu.et
 • Активно сотрудничает с UAEU (ОАЭ, член БРИКС+) с 2023 г
-• Город: кампус в г. Харамая (Восточный Харэр), почтовый ящик в Дыре-Дауэ; спутниковых проектов не найдено</t>
-        </is>
-      </c>
-      <c r="AH22" s="4" t="inlineStr">
+• Город: кампус в г. Харамая (Восточный Харэр), почтовый ящик в Дыре-Дауэ; спутниковых проектов не найдено
+• Рейтинги: Национального рейтинга с местами нет: МинОбр Эфиопии делит гос. вузы на категории (research / applied science / general), мест не публикует</t>
+        </is>
+      </c>
+      <c r="AI22" s="4" t="inlineStr">
         <is>
           <t>• Https://www.haramaya.edu.et
 • Https://www.haramaya.edu.et/president-of-the-university/
@@ -4677,15 +5090,16 @@
 • Https://www.haramaya.edu.et/haramaya-university-delegation-participates-in-qs-africa-forum-2026/
 • Haramaya Public and International Relations Directorate page
 • Https://www.wearetech.africa/en/fils-uk/news/tech/ethiopia-expands-space-program-with-2026-satellite-launch (general check: no Ethiopian university-built satellite)
-• Nanosats.csv (nation=Ethiopia: only ESSTI ET-SMART-RSS and cancelled AAiT ET-SAT)</t>
-        </is>
-      </c>
-      <c r="AI22" s="4" t="inlineStr">
+• Nanosats.csv (nation=Ethiopia: only ESSTI ET-SMART-RSS and cancelled AAiT ET-SAT)
+https://figshare.com/articles/preprint/Ranking_Web_of_Universities_webometrics_info_July_2026_edition/33062150</t>
+        </is>
+      </c>
+      <c r="AJ22" s="4" t="inlineStr">
         <is>
           <t>2026-10-05</t>
         </is>
       </c>
-      <c r="AJ22" s="4" t="inlineStr"/>
+      <c r="AK22" s="4" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="4" t="n">
@@ -4784,45 +5198,63 @@
           <t>President</t>
         </is>
       </c>
-      <c r="S23" s="4" t="inlineStr"/>
-      <c r="T23" s="4" t="inlineStr"/>
-      <c r="U23" s="4" t="inlineStr"/>
-      <c r="V23" s="4" t="n">
+      <c r="S23" s="4" t="inlineStr">
+        <is>
+          <t>QS2027: не в рейтинге</t>
+        </is>
+      </c>
+      <c r="T23" s="4" t="inlineStr">
+        <is>
+          <t>THE2027: не в рейтинге</t>
+        </is>
+      </c>
+      <c r="U23" s="4" t="inlineStr">
+        <is>
+          <t>нет общенационального рейтинга</t>
+        </is>
+      </c>
+      <c r="V23" s="4" t="inlineStr">
+        <is>
+          <t>3144</t>
+        </is>
+      </c>
+      <c r="W23" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="W23" s="4" t="inlineStr"/>
       <c r="X23" s="4" t="inlineStr"/>
       <c r="Y23" s="4" t="inlineStr"/>
       <c r="Z23" s="4" t="inlineStr"/>
       <c r="AA23" s="4" t="inlineStr"/>
       <c r="AB23" s="4" t="inlineStr"/>
-      <c r="AC23" s="4" t="n">
+      <c r="AC23" s="4" t="inlineStr"/>
+      <c r="AD23" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="AD23" s="8" t="inlineStr">
+      <c r="AE23" s="8" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="AE23" s="4" t="inlineStr">
+      <c r="AF23" s="4" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="AF23" s="4" t="inlineStr">
+      <c r="AG23" s="4" t="inlineStr">
         <is>
           <t>средняя</t>
         </is>
       </c>
-      <c r="AG23" s="4" t="inlineStr">
+      <c r="AH23" s="4" t="inlineStr">
         <is>
           <t>• Отдельного общего e-mail/e-mail президента нет; ccmd@hu.edu.et — ящик Public and International Relations Executive (указан и в подвале сайта как основной)
 • Глава офиса президента: Mr. Ayele Adato Yoma (только gmail, тел. +251 46 8871689)
 • Президент Dr. Chirotaw Ayele назначен ~окт. 2024 (ранее президент Dilla University)
-• Спутниковых проектов не найдено (быстрая проверка)</t>
-        </is>
-      </c>
-      <c r="AH23" s="4" t="inlineStr">
+• Спутниковых проектов не найдено (быстрая проверка)
+• Рейтинги: Национального рейтинга с местами нет: МинОбр Эфиопии делит гос. вузы на категории (research / applied science / general), мест не публикует</t>
+        </is>
+      </c>
+      <c r="AI23" s="4" t="inlineStr">
         <is>
           <t>• Https://www.hu.edu.et
 • Https://www.hu.edu.et/message-from-the-president
@@ -4830,15 +5262,16 @@
 • Https://www.hu.edu.et/president-office
 • Https://www.hu.edu.et/contact-us
 • Https://www.wearetech.africa/en/fils-uk/news/tech/ethiopia-expands-space-program-with-2026-satellite-launch (general check: no Ethiopian university-built satellite)
-• Nanosats.csv (nation=Ethiopia: only ESSTI ET-SMART-RSS and cancelled AAiT ET-SAT)</t>
-        </is>
-      </c>
-      <c r="AI23" s="4" t="inlineStr">
+• Nanosats.csv (nation=Ethiopia: only ESSTI ET-SMART-RSS and cancelled AAiT ET-SAT)
+https://figshare.com/articles/preprint/Ranking_Web_of_Universities_webometrics_info_July_2026_edition/33062150</t>
+        </is>
+      </c>
+      <c r="AJ23" s="4" t="inlineStr">
         <is>
           <t>2026-10-05</t>
         </is>
       </c>
-      <c r="AJ23" s="4" t="inlineStr"/>
+      <c r="AK23" s="4" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="4" t="n">
@@ -4933,45 +5366,63 @@
           <t>President</t>
         </is>
       </c>
-      <c r="S24" s="4" t="inlineStr"/>
-      <c r="T24" s="4" t="inlineStr"/>
-      <c r="U24" s="4" t="inlineStr"/>
-      <c r="V24" s="4" t="n">
+      <c r="S24" s="4" t="inlineStr">
+        <is>
+          <t>QS2027: не в рейтинге</t>
+        </is>
+      </c>
+      <c r="T24" s="4" t="inlineStr">
+        <is>
+          <t>THE2027: не в рейтинге</t>
+        </is>
+      </c>
+      <c r="U24" s="4" t="inlineStr">
+        <is>
+          <t>нет общенационального рейтинга</t>
+        </is>
+      </c>
+      <c r="V24" s="4" t="inlineStr">
+        <is>
+          <t>нет в опубл. списке</t>
+        </is>
+      </c>
+      <c r="W24" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="W24" s="4" t="inlineStr"/>
       <c r="X24" s="4" t="inlineStr"/>
       <c r="Y24" s="4" t="inlineStr"/>
       <c r="Z24" s="4" t="inlineStr"/>
       <c r="AA24" s="4" t="inlineStr"/>
       <c r="AB24" s="4" t="inlineStr"/>
-      <c r="AC24" s="4" t="n">
+      <c r="AC24" s="4" t="inlineStr"/>
+      <c r="AD24" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="AD24" s="8" t="inlineStr">
+      <c r="AE24" s="8" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="AE24" s="4" t="inlineStr">
+      <c r="AF24" s="4" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="AF24" s="4" t="inlineStr">
+      <c r="AG24" s="4" t="inlineStr">
         <is>
           <t>средняя</t>
         </is>
       </c>
-      <c r="AG24" s="4" t="inlineStr">
+      <c r="AH24" s="4" t="inlineStr">
         <is>
           <t>• Спутников на орбите не найдено (проверка: nanosats.csv и поиск 'Ethiopian university CubeSat launched', окт. 2026)
 • Президент Dr. Gardachew Worku (доцент) — на странице офиса президента; его имя встречается в новостях сайта май–июнь 2026
 • Международными связями ведает Управление по связям с общественностью и международным отношениям (руководитель Belayneh Agumas, тел. +251 918 058 583, только личный gmail) — официального e-mail отдела нет; использовать общий адрес
-• Второй телефон: +251 58 227 1674; почтовый ящик не подтверждён (на странице контактов в поле 'Fax' указано '40')</t>
-        </is>
-      </c>
-      <c r="AH24" s="4" t="inlineStr">
+• Второй телефон: +251 58 227 1674; почтовый ящик не подтверждён (на странице контактов в поле 'Fax' указано '40')
+• Рейтинги: Национального рейтинга с местами нет: МинОбр Эфиопии делит гос. вузы на категории (research / applied science / general), мест не публикует</t>
+        </is>
+      </c>
+      <c r="AI24" s="4" t="inlineStr">
         <is>
           <t>• Https://www.inu.edu.et/
 • Https://www.inu.edu.et/president/
@@ -4980,12 +5431,12 @@
 • Https://www.inu.edu.et/advanced-science-and-research-laboratory-inaugurated-at-injibara-university/</t>
         </is>
       </c>
-      <c r="AI24" s="4" t="inlineStr">
+      <c r="AJ24" s="4" t="inlineStr">
         <is>
           <t>2026-10-05</t>
         </is>
       </c>
-      <c r="AJ24" s="4" t="inlineStr"/>
+      <c r="AK24" s="4" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="4" t="n">
@@ -5048,41 +5499,51 @@
           <t>President</t>
         </is>
       </c>
-      <c r="S25" s="4" t="inlineStr"/>
-      <c r="T25" s="4" t="inlineStr"/>
+      <c r="S25" s="4" t="inlineStr">
+        <is>
+          <t>QS2027: не в рейтинге</t>
+        </is>
+      </c>
+      <c r="T25" s="4" t="inlineStr">
+        <is>
+          <t>THE2027: не в рейтинге</t>
+        </is>
+      </c>
       <c r="U25" s="4" t="inlineStr"/>
-      <c r="V25" s="4" t="n">
+      <c r="V25" s="4" t="inlineStr"/>
+      <c r="W25" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="W25" s="4" t="inlineStr"/>
       <c r="X25" s="4" t="inlineStr"/>
       <c r="Y25" s="4" t="inlineStr"/>
       <c r="Z25" s="4" t="inlineStr"/>
       <c r="AA25" s="4" t="inlineStr"/>
       <c r="AB25" s="4" t="inlineStr"/>
-      <c r="AC25" s="4" t="n">
+      <c r="AC25" s="4" t="inlineStr"/>
+      <c r="AD25" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="AD25" s="8" t="inlineStr">
+      <c r="AE25" s="8" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="AE25" s="4" t="inlineStr"/>
-      <c r="AF25" s="4" t="inlineStr">
+      <c r="AF25" s="4" t="inlineStr"/>
+      <c r="AG25" s="4" t="inlineStr">
         <is>
           <t>низкая</t>
         </is>
       </c>
-      <c r="AG25" s="4" t="inlineStr">
+      <c r="AH25" s="4" t="inlineStr">
         <is>
           <t>• Официальный сайт jju.edu.et заблокирован для нашего IP (редирект на страницу блокировки хостинга) — контакты и руководство не проверены; требуется ручная проверка
 • В Википедии (данные 2022 г.) президентом указан Dr. Bashir Abdulahi Mohamed — для 2026 не подтверждено, поэтому поле оставлено пустым
 • Сомалийский регион; спутниковых проектов не найдено
-• Перепроверка: 04.10.2026: jju.edu.et по-прежнему перенаправляет на страницу блокировки хостинга (technobros.au/blocked.html); данные не изменены</t>
-        </is>
-      </c>
-      <c r="AH25" s="4" t="inlineStr">
+• Перепроверка: 04.10.2026: jju.edu.et по-прежнему перенаправляет на страницу блокировки хостинга (technobros.au/blocked.html); данные не изменены
+• Ручная проверка: Рейтинги: QS 2027 — официальный файл данных topuniversities.com (qs-rankings-data/en/4153156.txt), сверка 05.10.2026; THE 2027 — список THE World University Rankings 2027 (data/sources/the2027.json). Webometrics: webometrics.info не открывается (DNS) — не заполнено</t>
+        </is>
+      </c>
+      <c r="AI25" s="4" t="inlineStr">
         <is>
           <t>• Https://www.jju.edu.et (blocked: redirects to technobros.au/blocked.html from our network)
 • Https://en.wikipedia.org/wiki/Jijiga_University (2022 data only)
@@ -5090,12 +5551,12 @@
 • Nanosats.csv (nation=Ethiopia: only ESSTI ET-SMART-RSS and cancelled AAiT ET-SAT)</t>
         </is>
       </c>
-      <c r="AI25" s="4" t="inlineStr">
+      <c r="AJ25" s="4" t="inlineStr">
         <is>
           <t>2026-10-05</t>
         </is>
       </c>
-      <c r="AJ25" s="4" t="inlineStr"/>
+      <c r="AK25" s="4" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="4" t="n">
@@ -5190,59 +5651,78 @@
           <t>President</t>
         </is>
       </c>
-      <c r="S26" s="4" t="inlineStr"/>
-      <c r="T26" s="4" t="inlineStr"/>
-      <c r="U26" s="4" t="inlineStr"/>
-      <c r="V26" s="4" t="n">
+      <c r="S26" s="4" t="inlineStr">
+        <is>
+          <t>QS2027: не в рейтинге</t>
+        </is>
+      </c>
+      <c r="T26" s="4" t="inlineStr">
+        <is>
+          <t>THE2027: не в рейтинге</t>
+        </is>
+      </c>
+      <c r="U26" s="4" t="inlineStr">
+        <is>
+          <t>нет общенационального рейтинга</t>
+        </is>
+      </c>
+      <c r="V26" s="4" t="inlineStr">
+        <is>
+          <t>2187</t>
+        </is>
+      </c>
+      <c r="W26" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="W26" s="4" t="inlineStr"/>
       <c r="X26" s="4" t="inlineStr"/>
       <c r="Y26" s="4" t="inlineStr"/>
       <c r="Z26" s="4" t="inlineStr"/>
       <c r="AA26" s="4" t="inlineStr"/>
       <c r="AB26" s="4" t="inlineStr"/>
-      <c r="AC26" s="4" t="n">
+      <c r="AC26" s="4" t="inlineStr"/>
+      <c r="AD26" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="AD26" s="8" t="inlineStr">
+      <c r="AE26" s="8" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="AE26" s="4" t="inlineStr">
+      <c r="AF26" s="4" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="AF26" s="4" t="inlineStr">
+      <c r="AG26" s="4" t="inlineStr">
         <is>
           <t>средняя</t>
         </is>
       </c>
-      <c r="AG26" s="4" t="inlineStr">
+      <c r="AH26" s="4" t="inlineStr">
         <is>
           <t>• Спутников на орбите не найдено (проверка: nanosats.csv и поиск 'Ethiopian university CubeSat launched', окт. 2026)
 • Президент Dr. Dereje Engida (PhD, доцент) подтверждён новостью сайта от 23.09.2026; в новостях пишется также 'Engeda'; личный e-mail президента: dereje.engida@ju.edu.et
 • Ero@ju.edu.et — единственный общий адрес на сайте (страница контактов); отдельный e-mail международного отдела не опубликован
-• На странице 'Internationalization and Institutional Collaboration' для потенциальных международных партнёров указан Mr. Addisalem Taye (taye.addisalem@ju.edu.et); дата страницы неизвестна — актуальность не подтверждена</t>
-        </is>
-      </c>
-      <c r="AH26" s="4" t="inlineStr">
+• На странице 'Internationalization and Institutional Collaboration' для потенциальных международных партнёров указан Mr. Addisalem Taye (taye.addisalem@ju.edu.et); дата страницы неизвестна — актуальность не подтверждена
+• Рейтинги: Национального рейтинга с местами нет: МинОбр Эфиопии делит гос. вузы на категории (research / applied science / general), мест не публикует</t>
+        </is>
+      </c>
+      <c r="AI26" s="4" t="inlineStr">
         <is>
           <t>• Https://ju.edu.et/
 • Https://ju.edu.et/presidents-message/
 • Https://ju.edu.et/contact-us/
 • Https://ju.edu.et/internationalization-and-institutional-collaboration/
-• Https://ju.edu.et/jimma-university-president-outlines-vision-for-institutional-autonomy-and-global-impact-in-address-to-academic-staff/</t>
-        </is>
-      </c>
-      <c r="AI26" s="4" t="inlineStr">
+• Https://ju.edu.et/jimma-university-president-outlines-vision-for-institutional-autonomy-and-global-impact-in-address-to-academic-staff/
+https://figshare.com/articles/preprint/Ranking_Web_of_Universities_webometrics_info_July_2026_edition/33062150</t>
+        </is>
+      </c>
+      <c r="AJ26" s="4" t="inlineStr">
         <is>
           <t>2026-10-05</t>
         </is>
       </c>
-      <c r="AJ26" s="4" t="inlineStr"/>
+      <c r="AK26" s="4" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="4" t="n">
@@ -5341,46 +5821,64 @@
           <t>President</t>
         </is>
       </c>
-      <c r="S27" s="4" t="inlineStr"/>
-      <c r="T27" s="4" t="inlineStr"/>
-      <c r="U27" s="4" t="inlineStr"/>
-      <c r="V27" s="4" t="n">
+      <c r="S27" s="4" t="inlineStr">
+        <is>
+          <t>QS2027: не в рейтинге</t>
+        </is>
+      </c>
+      <c r="T27" s="4" t="inlineStr">
+        <is>
+          <t>THE2027: не в рейтинге</t>
+        </is>
+      </c>
+      <c r="U27" s="4" t="inlineStr">
+        <is>
+          <t>нет общенационального рейтинга</t>
+        </is>
+      </c>
+      <c r="V27" s="4" t="inlineStr">
+        <is>
+          <t>нет в опубл. списке</t>
+        </is>
+      </c>
+      <c r="W27" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="W27" s="4" t="inlineStr"/>
       <c r="X27" s="4" t="inlineStr"/>
       <c r="Y27" s="4" t="inlineStr"/>
       <c r="Z27" s="4" t="inlineStr"/>
       <c r="AA27" s="4" t="inlineStr"/>
       <c r="AB27" s="4" t="inlineStr"/>
-      <c r="AC27" s="4" t="n">
+      <c r="AC27" s="4" t="inlineStr"/>
+      <c r="AD27" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="AD27" s="8" t="inlineStr">
+      <c r="AE27" s="8" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="AE27" s="4" t="inlineStr">
+      <c r="AF27" s="4" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="AF27" s="4" t="inlineStr">
+      <c r="AG27" s="4" t="inlineStr">
         <is>
           <t>средняя</t>
         </is>
       </c>
-      <c r="AG27" s="4" t="inlineStr">
+      <c r="AH27" s="4" t="inlineStr">
         <is>
           <t>• Спутников на орбите не найдено (проверка: nanosats.csv и поиск 'Ethiopian university CubeSat launched', окт. 2026)
 • Университет использует название 'University of Kabridahar' и домен uok.edu.et (kdu.edu.et перенаправляет туда)
 • Президент Eng. Abdifetah Ahmed Rabi (abdifetah@uok.edu.et) — по странице президента, дата не указана; учёная степень не указана, обращение 'Eng.'
 • Email_international — личный адрес руководителя Управления по связям с общественностью и международным отношениям (Abdiladif Ahmed Olad); телефоны на странице контактов: +251 915 744 573, +251 911 303 733
-• Name_native на сомалийском — по общепринятому написанию, на сайте не подтверждено</t>
-        </is>
-      </c>
-      <c r="AH27" s="4" t="inlineStr">
+• Name_native на сомалийском — по общепринятому написанию, на сайте не подтверждено
+• Рейтинги: Национального рейтинга с местами нет: МинОбр Эфиопии делит гос. вузы на категории (research / applied science / general), мест не публикует</t>
+        </is>
+      </c>
+      <c r="AI27" s="4" t="inlineStr">
         <is>
           <t>• Https://uok.edu.et/
 • Https://uok.edu.et/administration/president/
@@ -5388,12 +5886,12 @@
 • Https://uok.edu.et/contact/</t>
         </is>
       </c>
-      <c r="AI27" s="4" t="inlineStr">
+      <c r="AJ27" s="4" t="inlineStr">
         <is>
           <t>2026-10-05</t>
         </is>
       </c>
-      <c r="AJ27" s="4" t="inlineStr"/>
+      <c r="AK27" s="4" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="4" t="n">
@@ -5464,54 +5962,64 @@
           <t>President</t>
         </is>
       </c>
-      <c r="S28" s="4" t="inlineStr"/>
-      <c r="T28" s="4" t="inlineStr"/>
+      <c r="S28" s="4" t="inlineStr">
+        <is>
+          <t>QS2027: не в рейтинге</t>
+        </is>
+      </c>
+      <c r="T28" s="4" t="inlineStr">
+        <is>
+          <t>THE2027: не в рейтинге</t>
+        </is>
+      </c>
       <c r="U28" s="4" t="inlineStr"/>
-      <c r="V28" s="4" t="n">
+      <c r="V28" s="4" t="inlineStr"/>
+      <c r="W28" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="W28" s="4" t="inlineStr"/>
       <c r="X28" s="4" t="inlineStr"/>
       <c r="Y28" s="4" t="inlineStr"/>
       <c r="Z28" s="4" t="inlineStr"/>
       <c r="AA28" s="4" t="inlineStr"/>
       <c r="AB28" s="4" t="inlineStr"/>
-      <c r="AC28" s="4" t="n">
+      <c r="AC28" s="4" t="inlineStr"/>
+      <c r="AD28" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="AD28" s="8" t="inlineStr">
+      <c r="AE28" s="8" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="AE28" s="4" t="inlineStr"/>
-      <c r="AF28" s="4" t="inlineStr">
+      <c r="AF28" s="4" t="inlineStr"/>
+      <c r="AG28" s="4" t="inlineStr">
         <is>
           <t>низкая</t>
         </is>
       </c>
-      <c r="AG28" s="4" t="inlineStr">
+      <c r="AH28" s="4" t="inlineStr">
         <is>
           <t>• Спутников на орбите не найдено (проверка: nanosats.csv и поиск 'Ethiopian university CubeSat launched', окт. 2026)
 • Сайт kue.edu.et недоступен (ошибка базы данных HTTP 500, 04.10.2026) — контакты и руководство не проверены
 • Поисковая выдача называет президентом Dr. Teshome Nekatibeb (teshome.nekatibeb@kue.edu.et) — НЕ подтверждено открытой страницей; по другим данным, прежний президент Dr. Berhanemeskel Tena перешёл в Madda Walabu University
 • Name_native и city — по общепринятым данным; университет педагогический (бывш. Kotebe Metropolitan University)
 • Повторная проверка 04.10.2026: kue.edu.et (страницы President's Message, Senate Members) — HTTP 500/сброс соединения; поисковая выдача по-прежнему указывает Dr. Teshome Nekatibeb как президента и Dr. Berhanemeskel Tena как основателя-президента 2021–2026
-• Перепроверка: Сайт kue.edu.et по-прежнему недоступен (HTTP 500/сброс, 04.10.2026); данные не изменены — президент (по выдаче Dr. Teshome Nekatibeb) не подтверждён</t>
-        </is>
-      </c>
-      <c r="AH28" s="4" t="inlineStr">
+• Перепроверка: Сайт kue.edu.et по-прежнему недоступен (HTTP 500/сброс, 04.10.2026); данные не изменены — президент (по выдаче Dr. Teshome Nekatibeb) не подтверждён
+• Ручная проверка: Рейтинги: QS 2027 — официальный файл данных topuniversities.com (qs-rankings-data/en/4153156.txt), сверка 05.10.2026; THE 2027 — список THE World University Rankings 2027 (data/sources/the2027.json). Webometrics: webometrics.info не открывается (DNS) — не заполнено</t>
+        </is>
+      </c>
+      <c r="AI28" s="4" t="inlineStr">
         <is>
           <t>• Https://kue.edu.et (HTTP 500 database error / connection reset, Oct 2026)
 • Https://kue.edu.et/president-2/ (unreachable)</t>
         </is>
       </c>
-      <c r="AI28" s="4" t="inlineStr">
+      <c r="AJ28" s="4" t="inlineStr">
         <is>
           <t>2026-10-05</t>
         </is>
       </c>
-      <c r="AJ28" s="4" t="inlineStr"/>
+      <c r="AK28" s="4" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="4" t="n">
@@ -5587,42 +6095,52 @@
           <t>President</t>
         </is>
       </c>
-      <c r="S29" s="4" t="inlineStr"/>
-      <c r="T29" s="4" t="inlineStr"/>
+      <c r="S29" s="4" t="inlineStr">
+        <is>
+          <t>QS2027: не в рейтинге</t>
+        </is>
+      </c>
+      <c r="T29" s="4" t="inlineStr">
+        <is>
+          <t>THE2027: не в рейтинге</t>
+        </is>
+      </c>
       <c r="U29" s="4" t="inlineStr"/>
-      <c r="V29" s="4" t="n">
+      <c r="V29" s="4" t="inlineStr"/>
+      <c r="W29" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="W29" s="4" t="inlineStr"/>
       <c r="X29" s="4" t="inlineStr"/>
       <c r="Y29" s="4" t="inlineStr"/>
       <c r="Z29" s="4" t="inlineStr"/>
       <c r="AA29" s="4" t="inlineStr"/>
       <c r="AB29" s="4" t="inlineStr"/>
-      <c r="AC29" s="4" t="n">
+      <c r="AC29" s="4" t="inlineStr"/>
+      <c r="AD29" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="AD29" s="8" t="inlineStr">
+      <c r="AE29" s="8" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="AE29" s="4" t="inlineStr"/>
-      <c r="AF29" s="4" t="inlineStr">
+      <c r="AF29" s="4" t="inlineStr"/>
+      <c r="AG29" s="4" t="inlineStr">
         <is>
           <t>низкая</t>
         </is>
       </c>
-      <c r="AG29" s="4" t="inlineStr">
+      <c r="AH29" s="4" t="inlineStr">
         <is>
           <t>• Спутников на орбите не найдено (проверка: nanosats.csv и поиск 'Ethiopian university CubeSat launched', окт. 2026)
 • Сайт — SPA; его API (api.maddauni.online) возвращает 502, поэтому страницы президента, контактов и Директората исследований, интернационализации и партнёрств не открылись
 • Президент Dr. Berhanemeskel Tena (PhD) — по поисковому индексу официальной страницы mwu.edu.et/administration/president и Википедии (назначен в 2024 г., ранее — основатель-президент Kotebe University of Education); сам текст страницы не просмотрен — проверить
 • E-mail и телефон не подтверждены; в структуре сайта есть 'Research Internationalization and Partnership Directorate'
-• Перепроверка: Сайт mwu.edu.et (SPA) снова не отдал данные: API api.maddauni.online отвечает 502, в JS-бандле контактов нет; данные не изменены (04.10.2026)</t>
-        </is>
-      </c>
-      <c r="AH29" s="4" t="inlineStr">
+• Перепроверка: Сайт mwu.edu.et (SPA) снова не отдал данные: API api.maddauni.online отвечает 502, в JS-бандле контактов нет; данные не изменены (04.10.2026)
+• Ручная проверка: Рейтинги: QS 2027 — официальный файл данных topuniversities.com (qs-rankings-data/en/4153156.txt), сверка 05.10.2026; THE 2027 — список THE World University Rankings 2027 (data/sources/the2027.json). Webometrics: webometrics.info не открывается (DNS) — не заполнено</t>
+        </is>
+      </c>
+      <c r="AI29" s="4" t="inlineStr">
         <is>
           <t>• Https://mwu.edu.et/
 • Https://mwu.edu.et/data/page-routes.json
@@ -5630,12 +6148,12 @@
 • Https://en.wikipedia.org/wiki/Madda_Walabu_University</t>
         </is>
       </c>
-      <c r="AI29" s="4" t="inlineStr">
+      <c r="AJ29" s="4" t="inlineStr">
         <is>
           <t>2026-10-05</t>
         </is>
       </c>
-      <c r="AJ29" s="4" t="inlineStr"/>
+      <c r="AK29" s="4" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="4" t="n">
@@ -5734,45 +6252,63 @@
           <t>President</t>
         </is>
       </c>
-      <c r="S30" s="4" t="inlineStr"/>
-      <c r="T30" s="4" t="inlineStr"/>
-      <c r="U30" s="4" t="inlineStr"/>
-      <c r="V30" s="4" t="n">
+      <c r="S30" s="4" t="inlineStr">
+        <is>
+          <t>QS2027: не в рейтинге</t>
+        </is>
+      </c>
+      <c r="T30" s="4" t="inlineStr">
+        <is>
+          <t>THE2027: не в рейтинге</t>
+        </is>
+      </c>
+      <c r="U30" s="4" t="inlineStr">
+        <is>
+          <t>нет общенационального рейтинга</t>
+        </is>
+      </c>
+      <c r="V30" s="4" t="inlineStr">
+        <is>
+          <t>нет в опубл. списке</t>
+        </is>
+      </c>
+      <c r="W30" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="W30" s="4" t="inlineStr"/>
       <c r="X30" s="4" t="inlineStr"/>
       <c r="Y30" s="4" t="inlineStr"/>
       <c r="Z30" s="4" t="inlineStr"/>
       <c r="AA30" s="4" t="inlineStr"/>
       <c r="AB30" s="4" t="inlineStr"/>
-      <c r="AC30" s="4" t="n">
+      <c r="AC30" s="4" t="inlineStr"/>
+      <c r="AD30" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="AD30" s="8" t="inlineStr">
+      <c r="AE30" s="8" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="AE30" s="4" t="inlineStr">
+      <c r="AF30" s="4" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="AF30" s="4" t="inlineStr">
+      <c r="AG30" s="4" t="inlineStr">
         <is>
           <t>средняя</t>
         </is>
       </c>
-      <c r="AG30" s="4" t="inlineStr">
+      <c r="AH30" s="4" t="inlineStr">
         <is>
           <t>• Официальное название — Mattu University; на сайте используются два почтовых домена: meu.edu.et и mau.edu.et (у mau.edu.et действующая MX-запись Microsoft 365)
 • Директор Research, Internationalization Relations and Partnership Directorate — Dr. Tesfalem Atnafu (drtesfa@mau.edu.et, тел. +251 910 499 556); PIR Executive — Mr. Tegegn Demisse (pre@mau.edu.et)
 • Дата страницы президента не указана — актуальность на 2026 не подтверждена датированной новостью
-• Спутниковых проектов не найдено</t>
-        </is>
-      </c>
-      <c r="AH30" s="4" t="inlineStr">
+• Спутниковых проектов не найдено
+• Рейтинги: Национального рейтинга с местами нет: МинОбр Эфиопии делит гос. вузы на категории (research / applied science / general), мест не публикует</t>
+        </is>
+      </c>
+      <c r="AI30" s="4" t="inlineStr">
         <is>
           <t>• Https://www.meu.edu.et
 • Https://www.meu.edu.et/menu/president-office
@@ -5783,12 +6319,12 @@
 • Nanosats.csv (nation=Ethiopia: only ESSTI ET-SMART-RSS and cancelled AAiT ET-SAT)</t>
         </is>
       </c>
-      <c r="AI30" s="4" t="inlineStr">
+      <c r="AJ30" s="4" t="inlineStr">
         <is>
           <t>2026-10-05</t>
         </is>
       </c>
-      <c r="AJ30" s="4" t="inlineStr"/>
+      <c r="AK30" s="4" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="4" t="n">
@@ -5883,45 +6419,63 @@
           <t>President</t>
         </is>
       </c>
-      <c r="S31" s="4" t="inlineStr"/>
-      <c r="T31" s="4" t="inlineStr"/>
-      <c r="U31" s="4" t="inlineStr"/>
-      <c r="V31" s="4" t="n">
+      <c r="S31" s="4" t="inlineStr">
+        <is>
+          <t>QS2027: не в рейтинге</t>
+        </is>
+      </c>
+      <c r="T31" s="4" t="inlineStr">
+        <is>
+          <t>THE2027: не в рейтинге</t>
+        </is>
+      </c>
+      <c r="U31" s="4" t="inlineStr">
+        <is>
+          <t>нет общенационального рейтинга</t>
+        </is>
+      </c>
+      <c r="V31" s="4" t="inlineStr">
+        <is>
+          <t>нет в опубл. списке</t>
+        </is>
+      </c>
+      <c r="W31" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="W31" s="4" t="inlineStr"/>
       <c r="X31" s="4" t="inlineStr"/>
       <c r="Y31" s="4" t="inlineStr"/>
       <c r="Z31" s="4" t="inlineStr"/>
       <c r="AA31" s="4" t="inlineStr"/>
       <c r="AB31" s="4" t="inlineStr"/>
-      <c r="AC31" s="4" t="n">
+      <c r="AC31" s="4" t="inlineStr"/>
+      <c r="AD31" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="AD31" s="8" t="inlineStr">
+      <c r="AE31" s="8" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="AE31" s="4" t="inlineStr">
+      <c r="AF31" s="4" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="AF31" s="4" t="inlineStr">
+      <c r="AG31" s="4" t="inlineStr">
         <is>
           <t>средняя</t>
         </is>
       </c>
-      <c r="AG31" s="4" t="inlineStr">
+      <c r="AH31" s="4" t="inlineStr">
         <is>
           <t>• Спутников на орбите не найдено (проверка: nanosats.csv и поиск 'Ethiopian university CubeSat launched', окт. 2026)
 • Президент Dr. Wako Geda (PhD) упомянут в новости сайта, опубликованной 03.06.2026 (мероприятие 17.09.2018 по эфиопскому календарю ≈ май 2026); личный e-mail: wakogeda@mtu.edu.et
 • Отдельный международный отдел и его e-mail на сайте не найдены; использовать info@mtu.edu.et
-• Кампус Тепи: P.O. Box 121, тел. +251 47 556 1837</t>
-        </is>
-      </c>
-      <c r="AH31" s="4" t="inlineStr">
+• Кампус Тепи: P.O. Box 121, тел. +251 47 556 1837
+• Рейтинги: Национального рейтинга с местами нет: МинОбр Эфиопии делит гос. вузы на категории (research / applied science / general), мест не публикует</t>
+        </is>
+      </c>
+      <c r="AI31" s="4" t="inlineStr">
         <is>
           <t>• Https://mtu.edu.et/
 • Https://mtu.edu.et/office-of-the-president/
@@ -5930,12 +6484,12 @@
 • Https://mtu.edu.et/mizan-tepi-university-held-a-policy-briefing-on-may-17-2018/</t>
         </is>
       </c>
-      <c r="AI31" s="4" t="inlineStr">
+      <c r="AJ31" s="4" t="inlineStr">
         <is>
           <t>2026-10-05</t>
         </is>
       </c>
-      <c r="AJ31" s="4" t="inlineStr"/>
+      <c r="AK31" s="4" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="4" t="n">
@@ -6030,57 +6584,75 @@
           <t>President</t>
         </is>
       </c>
-      <c r="S32" s="4" t="inlineStr"/>
-      <c r="T32" s="4" t="inlineStr"/>
-      <c r="U32" s="4" t="inlineStr"/>
-      <c r="V32" s="4" t="n">
+      <c r="S32" s="4" t="inlineStr">
+        <is>
+          <t>QS2027: не в рейтинге</t>
+        </is>
+      </c>
+      <c r="T32" s="4" t="inlineStr">
+        <is>
+          <t>THE2027: не в рейтинге</t>
+        </is>
+      </c>
+      <c r="U32" s="4" t="inlineStr">
+        <is>
+          <t>нет общенационального рейтинга</t>
+        </is>
+      </c>
+      <c r="V32" s="4" t="inlineStr">
+        <is>
+          <t>нет в опубл. списке</t>
+        </is>
+      </c>
+      <c r="W32" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="W32" s="4" t="inlineStr"/>
       <c r="X32" s="4" t="inlineStr"/>
       <c r="Y32" s="4" t="inlineStr"/>
       <c r="Z32" s="4" t="inlineStr"/>
       <c r="AA32" s="4" t="inlineStr"/>
       <c r="AB32" s="4" t="inlineStr"/>
-      <c r="AC32" s="4" t="n">
+      <c r="AC32" s="4" t="inlineStr"/>
+      <c r="AD32" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="AD32" s="8" t="inlineStr">
+      <c r="AE32" s="8" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="AE32" s="4" t="inlineStr">
+      <c r="AF32" s="4" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="AF32" s="4" t="inlineStr">
+      <c r="AG32" s="4" t="inlineStr">
         <is>
           <t>средняя</t>
         </is>
       </c>
-      <c r="AG32" s="4" t="inlineStr">
+      <c r="AH32" s="4" t="inlineStr">
         <is>
           <t>• Спутников на орбите не найдено (проверка: nanosats.csv и поиск 'Ethiopian university CubeSat launched', окт. 2026)
 • Президент Prof. Muktar Mohammed (PhD) указан на главной странице сайта (окт. 2026); датированного подтверждения в новостях не найдено
 • Есть Директорат по связям с общественностью и международным отношениям при президенте, но его e-mail/руководитель не опубликованы
-• Альтернативный телефон на странице президента: +251 930 313 005; name_native на языке оромо — по общепринятому написанию, не с сайта</t>
-        </is>
-      </c>
-      <c r="AH32" s="4" t="inlineStr">
+• Альтернативный телефон на странице президента: +251 930 313 005; name_native на языке оромо — по общепринятому написанию, не с сайта
+• Рейтинги: Национального рейтинга с местами нет: МинОбр Эфиопии делит гос. вузы на категории (research / applied science / general), мест не публикует</t>
+        </is>
+      </c>
+      <c r="AI32" s="4" t="inlineStr">
         <is>
           <t>• Https://obu.edu.et/
 • Https://obu.edu.et/?page_id=2295
 • Https://obu.edu.et/?page_id=3905</t>
         </is>
       </c>
-      <c r="AI32" s="4" t="inlineStr">
+      <c r="AJ32" s="4" t="inlineStr">
         <is>
           <t>2026-10-05</t>
         </is>
       </c>
-      <c r="AJ32" s="4" t="inlineStr"/>
+      <c r="AK32" s="4" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="4" t="n">
@@ -6179,46 +6751,64 @@
           <t>President</t>
         </is>
       </c>
-      <c r="S33" s="4" t="inlineStr"/>
-      <c r="T33" s="4" t="inlineStr"/>
-      <c r="U33" s="4" t="inlineStr"/>
-      <c r="V33" s="4" t="n">
+      <c r="S33" s="4" t="inlineStr">
+        <is>
+          <t>QS2027: не в рейтинге</t>
+        </is>
+      </c>
+      <c r="T33" s="4" t="inlineStr">
+        <is>
+          <t>THE2027: не в рейтинге</t>
+        </is>
+      </c>
+      <c r="U33" s="4" t="inlineStr">
+        <is>
+          <t>нет общенационального рейтинга</t>
+        </is>
+      </c>
+      <c r="V33" s="4" t="inlineStr">
+        <is>
+          <t>нет в опубл. списке</t>
+        </is>
+      </c>
+      <c r="W33" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="W33" s="4" t="inlineStr"/>
       <c r="X33" s="4" t="inlineStr"/>
       <c r="Y33" s="4" t="inlineStr"/>
       <c r="Z33" s="4" t="inlineStr"/>
       <c r="AA33" s="4" t="inlineStr"/>
       <c r="AB33" s="4" t="inlineStr"/>
-      <c r="AC33" s="4" t="n">
+      <c r="AC33" s="4" t="inlineStr"/>
+      <c r="AD33" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="AD33" s="8" t="inlineStr">
+      <c r="AE33" s="8" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="AE33" s="4" t="inlineStr">
+      <c r="AF33" s="4" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="AF33" s="4" t="inlineStr">
+      <c r="AG33" s="4" t="inlineStr">
         <is>
           <t>средняя</t>
         </is>
       </c>
-      <c r="AG33" s="4" t="inlineStr">
+      <c r="AH33" s="4" t="inlineStr">
         <is>
           <t>• ВНИМАНИЕ: Тыграй (юг, г. Майчеу). С 9 сент. 2026 МинОбр приостановило зачисление и временно переводит студентов Raya University в другие вузы из-за небезопасности; последние новости на сайте — дек. 2025
 • ВНИМАНИЕ: сайт, по-видимому, частично скомпрометирован — при запросе с некоторыми user-agent www.rayu.edu.et отдаёт индонезийский спам (онлайн-казино); с обычным браузером открывается нормальный сайт
 • Public &amp; International Relations Executive Officer — Dr. Gessesse Nigusse Abebe (gessessenigusse@rayu.edu.et, +251 934 979 939); ящик офиса PRD@rayu.edu.et (Block 04, F-01, R-104)
 • Написание имени президента на сайте варьируется: Tadesse Dejenie / Dejene / Dejennie; глава офиса президента — Mr. HaileKiros Kebede (po@rayu.edu.et)
-• Спутниковых проектов не найдено</t>
-        </is>
-      </c>
-      <c r="AH33" s="4" t="inlineStr">
+• Спутниковых проектов не найдено
+• Рейтинги: Национального рейтинга с местами нет: МинОбр Эфиопии делит гос. вузы на категории (research / applied science / general), мест не публикует</t>
+        </is>
+      </c>
+      <c r="AI33" s="4" t="inlineStr">
         <is>
           <t>• Https://www.rayu.edu.et
 • Https://www.rayu.edu.et/contact-us-page/
@@ -6231,12 +6821,12 @@
 • Nanosats.csv (nation=Ethiopia: only ESSTI ET-SMART-RSS and cancelled AAiT ET-SAT)</t>
         </is>
       </c>
-      <c r="AI33" s="4" t="inlineStr">
+      <c r="AJ33" s="4" t="inlineStr">
         <is>
           <t>2026-10-05</t>
         </is>
       </c>
-      <c r="AJ33" s="4" t="inlineStr"/>
+      <c r="AK33" s="4" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="4" t="n">
@@ -6335,44 +6925,62 @@
           <t>President</t>
         </is>
       </c>
-      <c r="S34" s="4" t="inlineStr"/>
-      <c r="T34" s="4" t="inlineStr"/>
-      <c r="U34" s="4" t="inlineStr"/>
-      <c r="V34" s="4" t="n">
+      <c r="S34" s="4" t="inlineStr">
+        <is>
+          <t>QS2027: не в рейтинге</t>
+        </is>
+      </c>
+      <c r="T34" s="4" t="inlineStr">
+        <is>
+          <t>THE2027: не в рейтинге</t>
+        </is>
+      </c>
+      <c r="U34" s="4" t="inlineStr">
+        <is>
+          <t>нет общенационального рейтинга</t>
+        </is>
+      </c>
+      <c r="V34" s="4" t="inlineStr">
+        <is>
+          <t>нет в опубл. списке</t>
+        </is>
+      </c>
+      <c r="W34" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="W34" s="4" t="inlineStr"/>
       <c r="X34" s="4" t="inlineStr"/>
       <c r="Y34" s="4" t="inlineStr"/>
       <c r="Z34" s="4" t="inlineStr"/>
       <c r="AA34" s="4" t="inlineStr"/>
       <c r="AB34" s="4" t="inlineStr"/>
-      <c r="AC34" s="4" t="n">
+      <c r="AC34" s="4" t="inlineStr"/>
+      <c r="AD34" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="AD34" s="8" t="inlineStr">
+      <c r="AE34" s="8" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="AE34" s="4" t="inlineStr">
+      <c r="AF34" s="4" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="AF34" s="4" t="inlineStr">
+      <c r="AG34" s="4" t="inlineStr">
         <is>
           <t>средняя</t>
         </is>
       </c>
-      <c r="AG34" s="4" t="inlineStr">
+      <c r="AH34" s="4" t="inlineStr">
         <is>
           <t>• Официальное написание на сайте — Salale University (SlU); город Фиче (Северная Шоа, Оромия)
 • Executive for Public and International Relations — Dr. Yeshimebet Bogale (личный рабочий адрес yeshimebet_bogale@slu.edu.et, тел. +251 911 042 982); отдельного ящика международного офиса нет; также есть contact@slu.edu.et
-• Спутниковых проектов не найдено</t>
-        </is>
-      </c>
-      <c r="AH34" s="4" t="inlineStr">
+• Спутниковых проектов не найдено
+• Рейтинги: Национального рейтинга с местами нет: МинОбр Эфиопии делит гос. вузы на категории (research / applied science / general), мест не публикует</t>
+        </is>
+      </c>
+      <c r="AI34" s="4" t="inlineStr">
         <is>
           <t>• Https://slu.edu.et
 • Https://slu.edu.et/SLU_WEB/president-message.php
@@ -6382,12 +6990,12 @@
 • Nanosats.csv (nation=Ethiopia: only ESSTI ET-SMART-RSS and cancelled AAiT ET-SAT)</t>
         </is>
       </c>
-      <c r="AI34" s="4" t="inlineStr">
+      <c r="AJ34" s="4" t="inlineStr">
         <is>
           <t>2026-10-05</t>
         </is>
       </c>
-      <c r="AJ34" s="4" t="inlineStr"/>
+      <c r="AK34" s="4" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="4" t="n">
@@ -6485,44 +7093,62 @@
           <t>President</t>
         </is>
       </c>
-      <c r="S35" s="4" t="inlineStr"/>
-      <c r="T35" s="4" t="inlineStr"/>
-      <c r="U35" s="4" t="inlineStr"/>
-      <c r="V35" s="4" t="n">
+      <c r="S35" s="4" t="inlineStr">
+        <is>
+          <t>QS2027: не в рейтинге</t>
+        </is>
+      </c>
+      <c r="T35" s="4" t="inlineStr">
+        <is>
+          <t>THE2027: не в рейтинге</t>
+        </is>
+      </c>
+      <c r="U35" s="4" t="inlineStr">
+        <is>
+          <t>нет общенационального рейтинга</t>
+        </is>
+      </c>
+      <c r="V35" s="4" t="inlineStr">
+        <is>
+          <t>нет в опубл. списке</t>
+        </is>
+      </c>
+      <c r="W35" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="W35" s="4" t="inlineStr"/>
       <c r="X35" s="4" t="inlineStr"/>
       <c r="Y35" s="4" t="inlineStr"/>
       <c r="Z35" s="4" t="inlineStr"/>
       <c r="AA35" s="4" t="inlineStr"/>
       <c r="AB35" s="4" t="inlineStr"/>
-      <c r="AC35" s="4" t="n">
+      <c r="AC35" s="4" t="inlineStr"/>
+      <c r="AD35" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="AD35" s="8" t="inlineStr">
+      <c r="AE35" s="8" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="AE35" s="4" t="inlineStr">
+      <c r="AF35" s="4" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="AF35" s="4" t="inlineStr">
+      <c r="AG35" s="4" t="inlineStr">
         <is>
           <t>средняя</t>
         </is>
       </c>
-      <c r="AG35" s="4" t="inlineStr">
+      <c r="AH35" s="4" t="inlineStr">
         <is>
           <t>• Ящик международных партнёрств intlpartnership@su.edu.et опубликован в разделе 'Important contacts'; имя руководителя офиса на сайте не найдено
 • Также опубликованы presidentoffice@su.edu.et (офис президента); телефон — мобильный номер, указанный на сайте
-• Регион Афар; есть Школа наук о Земле; спутниковых проектов не найдено</t>
-        </is>
-      </c>
-      <c r="AH35" s="4" t="inlineStr">
+• Регион Афар; есть Школа наук о Земле; спутниковых проектов не найдено
+• Рейтинги: Национального рейтинга с местами нет: МинОбр Эфиопии делит гос. вузы на категории (research / applied science / general), мест не публикует</t>
+        </is>
+      </c>
+      <c r="AI35" s="4" t="inlineStr">
         <is>
           <t>• Https://su.edu.et
 • Https://su.edu.et/contact-us/
@@ -6531,12 +7157,12 @@
 • Nanosats.csv (nation=Ethiopia: only ESSTI ET-SMART-RSS and cancelled AAiT ET-SAT)</t>
         </is>
       </c>
-      <c r="AI35" s="4" t="inlineStr">
+      <c r="AJ35" s="4" t="inlineStr">
         <is>
           <t>2026-10-05</t>
         </is>
       </c>
-      <c r="AJ35" s="4" t="inlineStr"/>
+      <c r="AK35" s="4" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="4" t="n">
@@ -6635,58 +7261,77 @@
           <t>President</t>
         </is>
       </c>
-      <c r="S36" s="4" t="inlineStr"/>
-      <c r="T36" s="4" t="inlineStr"/>
-      <c r="U36" s="4" t="inlineStr"/>
-      <c r="V36" s="4" t="n">
+      <c r="S36" s="4" t="inlineStr">
+        <is>
+          <t>QS2027: не в рейтинге</t>
+        </is>
+      </c>
+      <c r="T36" s="4" t="inlineStr">
+        <is>
+          <t>THE2027: не в рейтинге</t>
+        </is>
+      </c>
+      <c r="U36" s="4" t="inlineStr">
+        <is>
+          <t>нет общенационального рейтинга</t>
+        </is>
+      </c>
+      <c r="V36" s="4" t="inlineStr">
+        <is>
+          <t>1299</t>
+        </is>
+      </c>
+      <c r="W36" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="W36" s="4" t="inlineStr"/>
       <c r="X36" s="4" t="inlineStr"/>
       <c r="Y36" s="4" t="inlineStr"/>
       <c r="Z36" s="4" t="inlineStr"/>
       <c r="AA36" s="4" t="inlineStr"/>
       <c r="AB36" s="4" t="inlineStr"/>
-      <c r="AC36" s="4" t="n">
+      <c r="AC36" s="4" t="inlineStr"/>
+      <c r="AD36" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="AD36" s="8" t="inlineStr">
+      <c r="AE36" s="8" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="AE36" s="4" t="inlineStr">
+      <c r="AF36" s="4" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="AF36" s="4" t="inlineStr">
+      <c r="AG36" s="4" t="inlineStr">
         <is>
           <t>средняя</t>
         </is>
       </c>
-      <c r="AG36" s="4" t="inlineStr">
+      <c r="AH36" s="4" t="inlineStr">
         <is>
           <t>• Спутников на орбите не найдено (проверка: nanosats.csv и поиск 'Ethiopian university CubeSat launched', окт. 2026)
 • Президент Yechale Kebede, PhD — по странице 'President’s Message' на официальном сайте (дата страницы не указана); e-mail президента: yechale.kebede@uog.edu.et
 • Директорат международных связей и партнёрств создан как отдельное подразделение в ноябре 2024 г.; директор — Solomon Girma Yabowork, PhD, тел. +251 92 057 0919
-• Почтовый ящик 196 взят со страницы контактов (число '196' рядом с 'President Building') — проверить; общий тел. на странице контактов: +251 588 940 290</t>
-        </is>
-      </c>
-      <c r="AH36" s="4" t="inlineStr">
+• Почтовый ящик 196 взят со страницы контактов (число '196' рядом с 'President Building') — проверить; общий тел. на странице контактов: +251 588 940 290
+• Рейтинги: Национального рейтинга с местами нет: МинОбр Эфиопии делит гос. вузы на категории (research / applied science / general), мест не публикует</t>
+        </is>
+      </c>
+      <c r="AI36" s="4" t="inlineStr">
         <is>
           <t>• Https://uog.edu.et/
 • Https://uog.edu.et/presidents-message/
 • Https://uog.edu.et/contact-us/
-• Https://uog.edu.et/international-relations-and-partnerships-directorate/</t>
-        </is>
-      </c>
-      <c r="AI36" s="4" t="inlineStr">
+• Https://uog.edu.et/international-relations-and-partnerships-directorate/
+https://figshare.com/articles/preprint/Ranking_Web_of_Universities_webometrics_info_July_2026_edition/33062150</t>
+        </is>
+      </c>
+      <c r="AJ36" s="4" t="inlineStr">
         <is>
           <t>2026-10-05</t>
         </is>
       </c>
-      <c r="AJ36" s="4" t="inlineStr"/>
+      <c r="AK36" s="4" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="4" t="n">
@@ -6781,59 +7426,78 @@
           <t>President</t>
         </is>
       </c>
-      <c r="S37" s="4" t="inlineStr"/>
-      <c r="T37" s="4" t="inlineStr"/>
-      <c r="U37" s="4" t="inlineStr"/>
-      <c r="V37" s="4" t="n">
+      <c r="S37" s="4" t="inlineStr">
+        <is>
+          <t>QS2027: не в рейтинге</t>
+        </is>
+      </c>
+      <c r="T37" s="4" t="inlineStr">
+        <is>
+          <t>THE2027: не в рейтинге</t>
+        </is>
+      </c>
+      <c r="U37" s="4" t="inlineStr">
+        <is>
+          <t>нет общенационального рейтинга</t>
+        </is>
+      </c>
+      <c r="V37" s="4" t="inlineStr">
+        <is>
+          <t>5312</t>
+        </is>
+      </c>
+      <c r="W37" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="W37" s="4" t="inlineStr"/>
       <c r="X37" s="4" t="inlineStr"/>
       <c r="Y37" s="4" t="inlineStr"/>
       <c r="Z37" s="4" t="inlineStr"/>
       <c r="AA37" s="4" t="inlineStr"/>
       <c r="AB37" s="4" t="inlineStr"/>
-      <c r="AC37" s="4" t="n">
+      <c r="AC37" s="4" t="inlineStr"/>
+      <c r="AD37" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="AD37" s="8" t="inlineStr">
+      <c r="AE37" s="8" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="AE37" s="4" t="inlineStr">
+      <c r="AF37" s="4" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="AF37" s="4" t="inlineStr">
+      <c r="AG37" s="4" t="inlineStr">
         <is>
           <t>средняя</t>
         </is>
       </c>
-      <c r="AG37" s="4" t="inlineStr">
+      <c r="AH37" s="4" t="inlineStr">
         <is>
           <t>• Спутников на орбите не найдено (проверка: nanosats.csv и поиск 'Ethiopian university CubeSat launched', окт. 2026)
 • Президент Guchie Gulie Sulla (PhD) указан на странице 'Message from the President'; последнее датированное упоминание в новостях сайта — май 2024; более свежего подтверждения (2025–2026) не найдено
 • Личный e-mail президента: guchie.gulie@wsu.edu.et
-• При офисе президента есть Директорат международных связей, но его e-mail и руководитель на сайте не опубликованы; использовать общий адрес wsu@wsu.edu.et</t>
-        </is>
-      </c>
-      <c r="AH37" s="4" t="inlineStr">
+• При офисе президента есть Директорат международных связей, но его e-mail и руководитель на сайте не опубликованы; использовать общий адрес wsu@wsu.edu.et
+• Рейтинги: Национального рейтинга с местами нет: МинОбр Эфиопии делит гос. вузы на категории (research / applied science / general), мест не публикует</t>
+        </is>
+      </c>
+      <c r="AI37" s="4" t="inlineStr">
         <is>
           <t>• Https://www.wsu.edu.et/
 • Https://www.wsu.edu.et/pages/pres_mess-sm-kk
 • Https://www.wsu.edu.et/pages/adm_pres-sm-kk
 • Https://www.wsu.edu.et/news/3
-• Https://www.wsu.edu.et/boardmembers</t>
-        </is>
-      </c>
-      <c r="AI37" s="4" t="inlineStr">
+• Https://www.wsu.edu.et/boardmembers
+https://figshare.com/articles/preprint/Ranking_Web_of_Universities_webometrics_info_July_2026_edition/33062150</t>
+        </is>
+      </c>
+      <c r="AJ37" s="4" t="inlineStr">
         <is>
           <t>2026-10-05</t>
         </is>
       </c>
-      <c r="AJ37" s="4" t="inlineStr"/>
+      <c r="AK37" s="4" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="4" t="n">
@@ -6932,45 +7596,63 @@
           <t>President</t>
         </is>
       </c>
-      <c r="S38" s="4" t="inlineStr"/>
-      <c r="T38" s="4" t="inlineStr"/>
-      <c r="U38" s="4" t="inlineStr"/>
-      <c r="V38" s="4" t="n">
+      <c r="S38" s="4" t="inlineStr">
+        <is>
+          <t>QS2027: не в рейтинге</t>
+        </is>
+      </c>
+      <c r="T38" s="4" t="inlineStr">
+        <is>
+          <t>THE2027: не в рейтинге</t>
+        </is>
+      </c>
+      <c r="U38" s="4" t="inlineStr">
+        <is>
+          <t>нет общенационального рейтинга</t>
+        </is>
+      </c>
+      <c r="V38" s="4" t="inlineStr">
+        <is>
+          <t>нет в опубл. списке</t>
+        </is>
+      </c>
+      <c r="W38" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="W38" s="4" t="inlineStr"/>
       <c r="X38" s="4" t="inlineStr"/>
       <c r="Y38" s="4" t="inlineStr"/>
       <c r="Z38" s="4" t="inlineStr"/>
       <c r="AA38" s="4" t="inlineStr"/>
       <c r="AB38" s="4" t="inlineStr"/>
-      <c r="AC38" s="4" t="n">
+      <c r="AC38" s="4" t="inlineStr"/>
+      <c r="AD38" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="AD38" s="8" t="inlineStr">
+      <c r="AE38" s="8" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="AE38" s="4" t="inlineStr">
+      <c r="AF38" s="4" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="AF38" s="4" t="inlineStr">
+      <c r="AG38" s="4" t="inlineStr">
         <is>
           <t>средняя</t>
         </is>
       </c>
-      <c r="AG38" s="4" t="inlineStr">
+      <c r="AH38" s="4" t="inlineStr">
         <is>
           <t>• Спутников на орбите не найдено (проверка: nanosats.csv и поиск 'Ethiopian university CubeSat launched', окт. 2026)
 • Президент Dr. Anegagregn Gashaw Ferede (PhD) — по странице послания президента (дата не указана); личный e-mail: anegagregng@wldu.edu.et
 • Директорат исследований, международных связей и партнёрств (RIRP) создан при реорганизации 2024 г.; директор Dr. Fentaw Baye Adal, моб. +251 931 137 968
-• В исходном коде сайта встречается посторонний адрес admin@kingsteruni.edu (шаблон) — не использовать</t>
-        </is>
-      </c>
-      <c r="AH38" s="4" t="inlineStr">
+• В исходном коде сайта встречается посторонний адрес admin@kingsteruni.edu (шаблон) — не использовать
+• Рейтинги: Национального рейтинга с местами нет: МинОбр Эфиопии делит гос. вузы на категории (research / applied science / general), мест не публикует</t>
+        </is>
+      </c>
+      <c r="AI38" s="4" t="inlineStr">
         <is>
           <t>• Https://wldu.edu.et/
 • Https://wldu.edu.et/presidents-message/
@@ -6978,12 +7660,12 @@
 • Https://wldu.edu.et/contact/</t>
         </is>
       </c>
-      <c r="AI38" s="4" t="inlineStr">
+      <c r="AJ38" s="4" t="inlineStr">
         <is>
           <t>2026-10-05</t>
         </is>
       </c>
-      <c r="AJ38" s="4" t="inlineStr"/>
+      <c r="AK38" s="4" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="4" t="n">
@@ -7082,46 +7764,64 @@
           <t>President</t>
         </is>
       </c>
-      <c r="S39" s="4" t="inlineStr"/>
-      <c r="T39" s="4" t="inlineStr"/>
-      <c r="U39" s="4" t="inlineStr"/>
-      <c r="V39" s="4" t="n">
+      <c r="S39" s="4" t="inlineStr">
+        <is>
+          <t>QS2027: не в рейтинге</t>
+        </is>
+      </c>
+      <c r="T39" s="4" t="inlineStr">
+        <is>
+          <t>THE2027: не в рейтинге</t>
+        </is>
+      </c>
+      <c r="U39" s="4" t="inlineStr">
+        <is>
+          <t>нет общенационального рейтинга</t>
+        </is>
+      </c>
+      <c r="V39" s="4" t="inlineStr">
+        <is>
+          <t>нет в опубл. списке</t>
+        </is>
+      </c>
+      <c r="W39" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="W39" s="4" t="inlineStr"/>
       <c r="X39" s="4" t="inlineStr"/>
       <c r="Y39" s="4" t="inlineStr"/>
       <c r="Z39" s="4" t="inlineStr"/>
       <c r="AA39" s="4" t="inlineStr"/>
       <c r="AB39" s="4" t="inlineStr"/>
-      <c r="AC39" s="4" t="n">
+      <c r="AC39" s="4" t="inlineStr"/>
+      <c r="AD39" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="AD39" s="8" t="inlineStr">
+      <c r="AE39" s="8" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="AE39" s="4" t="inlineStr">
+      <c r="AF39" s="4" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="AF39" s="4" t="inlineStr">
+      <c r="AG39" s="4" t="inlineStr">
         <is>
           <t>средняя</t>
         </is>
       </c>
-      <c r="AG39" s="4" t="inlineStr">
+      <c r="AH39" s="4" t="inlineStr">
         <is>
           <t>• Спутников на орбите не найдено (проверка: nanosats.csv и поиск 'Ethiopian university CubeSat launched', окт. 2026)
 • Новый президент с июня 2026 г. (сменил Dr. Faris Delil, руководившего 6 лет); написание имени различается: Abdlmuhsin Hassen Alajib / Abdulemuhesin Hassen / Abdelmuhsin Hasen
 • Университет отнесён МО к категории 'прикладных наук' (applied sciences)
 • President.chiefhead@wku.edu.et — ящик руководителя офиса президента (Mr. Melesse Etifu Meranga, тел. +251 911 376 067); e-mail адреса декодированы из защищённой разметки сайта
-• Директор по исследованиям, международным связям и партнёрствам: Dr. Mitiku Tasisa Dinsa, тел. +251 913 835 518 (также mitiku1tasisa@gmail.com); тел. +251 11 322 0162 указан на странице офиса президента — проверить</t>
-        </is>
-      </c>
-      <c r="AH39" s="4" t="inlineStr">
+• Директор по исследованиям, международным связям и партнёрствам: Dr. Mitiku Tasisa Dinsa, тел. +251 913 835 518 (также mitiku1tasisa@gmail.com); тел. +251 11 322 0162 указан на странице офиса президента — проверить
+• Рейтинги: Национального рейтинга с местами нет: МинОбр Эфиопии делит гос. вузы на категории (research / applied science / general), мест не публикует</t>
+        </is>
+      </c>
+      <c r="AI39" s="4" t="inlineStr">
         <is>
           <t>• Https://www.wku.edu.et/
 • Https://www.wku.edu.et/index.php/en/about-us/presidents-message
@@ -7131,12 +7831,12 @@
 • Https://www.wku.edu.et/index.php/en/component/content/article/2026-06-11-16-24-56?catid=12</t>
         </is>
       </c>
-      <c r="AI39" s="4" t="inlineStr">
+      <c r="AJ39" s="4" t="inlineStr">
         <is>
           <t>2026-10-05</t>
         </is>
       </c>
-      <c r="AJ39" s="4" t="inlineStr"/>
+      <c r="AK39" s="4" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="4" t="n">
@@ -7231,44 +7931,62 @@
           <t>President</t>
         </is>
       </c>
-      <c r="S40" s="4" t="inlineStr"/>
-      <c r="T40" s="4" t="inlineStr"/>
-      <c r="U40" s="4" t="inlineStr"/>
-      <c r="V40" s="4" t="n">
+      <c r="S40" s="4" t="inlineStr">
+        <is>
+          <t>QS2027: не в рейтинге</t>
+        </is>
+      </c>
+      <c r="T40" s="4" t="inlineStr">
+        <is>
+          <t>THE2027: не в рейтинге</t>
+        </is>
+      </c>
+      <c r="U40" s="4" t="inlineStr">
+        <is>
+          <t>нет общенационального рейтинга</t>
+        </is>
+      </c>
+      <c r="V40" s="4" t="inlineStr">
+        <is>
+          <t>нет в опубл. списке</t>
+        </is>
+      </c>
+      <c r="W40" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="W40" s="4" t="inlineStr"/>
       <c r="X40" s="4" t="inlineStr"/>
       <c r="Y40" s="4" t="inlineStr"/>
       <c r="Z40" s="4" t="inlineStr"/>
       <c r="AA40" s="4" t="inlineStr"/>
       <c r="AB40" s="4" t="inlineStr"/>
-      <c r="AC40" s="4" t="n">
+      <c r="AC40" s="4" t="inlineStr"/>
+      <c r="AD40" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="AD40" s="8" t="inlineStr">
+      <c r="AE40" s="8" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="AE40" s="4" t="inlineStr">
+      <c r="AF40" s="4" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="AF40" s="4" t="inlineStr">
+      <c r="AG40" s="4" t="inlineStr">
         <is>
           <t>средняя</t>
         </is>
       </c>
-      <c r="AG40" s="4" t="inlineStr">
+      <c r="AH40" s="4" t="inlineStr">
         <is>
           <t>• ВНИМАНИЕ: 14.09.2026 университет объявил конкурс на должности президента и двух вице-президентов (директива МинОбр № 1146/2018 E.C.) — вероятна смена руководства; Dr. Tesfaye Lemma (Associate Professor) — президент на момент проверки
 • International Relations and Partnership Directorate (страница от 26.05.2026): тел. +251 917 660 150, Main Campus Administration Building; e-mail опубликован с опечаткой в домене — 'galatag@wollegauniveristy.edu.et' (и gmail galatagamachu1@gmail.com); имя директора не указано. Поэтому письмо — на info@wollegauniversity.edu.et
-• Оромия (западная часть) — возможны проблемы с безопасностью; спутниковых проектов не найдено</t>
-        </is>
-      </c>
-      <c r="AH40" s="4" t="inlineStr">
+• Оромия (западная часть) — возможны проблемы с безопасностью; спутниковых проектов не найдено
+• Рейтинги: Национального рейтинга с местами нет: МинОбр Эфиопии делит гос. вузы на категории (research / applied science / general), мест не публикует</t>
+        </is>
+      </c>
+      <c r="AI40" s="4" t="inlineStr">
         <is>
           <t>• Https://wollegauniversity.edu.et
 • Https://wollegauniversity.edu.et/index.php/gallery/president-office-2/international-relations-and-partnership-directorate (26 May 2026)
@@ -7277,12 +7995,12 @@
 • Nanosats.csv (nation=Ethiopia: only ESSTI ET-SMART-RSS and cancelled AAiT ET-SAT)</t>
         </is>
       </c>
-      <c r="AI40" s="4" t="inlineStr">
+      <c r="AJ40" s="4" t="inlineStr">
         <is>
           <t>2026-10-05</t>
         </is>
       </c>
-      <c r="AJ40" s="4" t="inlineStr"/>
+      <c r="AK40" s="4" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="4" t="n">
@@ -7376,62 +8094,81 @@
           <t>President</t>
         </is>
       </c>
-      <c r="S41" s="4" t="inlineStr"/>
-      <c r="T41" s="4" t="inlineStr"/>
-      <c r="U41" s="4" t="inlineStr"/>
-      <c r="V41" s="4" t="n">
+      <c r="S41" s="4" t="inlineStr">
+        <is>
+          <t>QS2027: не в рейтинге</t>
+        </is>
+      </c>
+      <c r="T41" s="4" t="inlineStr">
+        <is>
+          <t>THE2027: не в рейтинге</t>
+        </is>
+      </c>
+      <c r="U41" s="4" t="inlineStr">
+        <is>
+          <t>нет общенационального рейтинга</t>
+        </is>
+      </c>
+      <c r="V41" s="4" t="inlineStr">
+        <is>
+          <t>4470</t>
+        </is>
+      </c>
+      <c r="W41" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="W41" s="4" t="inlineStr"/>
       <c r="X41" s="4" t="inlineStr"/>
       <c r="Y41" s="4" t="inlineStr"/>
       <c r="Z41" s="4" t="inlineStr"/>
       <c r="AA41" s="4" t="inlineStr"/>
       <c r="AB41" s="4" t="inlineStr"/>
-      <c r="AC41" s="4" t="n">
+      <c r="AC41" s="4" t="inlineStr"/>
+      <c r="AD41" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="AD41" s="8" t="inlineStr">
+      <c r="AE41" s="8" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="AE41" s="4" t="inlineStr">
+      <c r="AF41" s="4" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="AF41" s="4" t="inlineStr">
+      <c r="AG41" s="4" t="inlineStr">
         <is>
           <t>средняя</t>
         </is>
       </c>
-      <c r="AG41" s="4" t="inlineStr">
+      <c r="AH41" s="4" t="inlineStr">
         <is>
           <t>• Страницы President Office и International Relation на сайте пустые — имя руководителя международного отдела и отдельный e-mail не опубликованы; письмо на общий адрес info@wu.edu.et
 • Номер почтового ящика (P.O. Box) на сайте не указан
 • Регион Амхара — возможны проблемы с безопасностью/связью
-• Спутниковых проектов не найдено</t>
-        </is>
-      </c>
-      <c r="AH41" s="4" t="inlineStr">
+• Спутниковых проектов не найдено
+• Рейтинги: Национального рейтинга с местами нет: МинОбр Эфиопии делит гос. вузы на категории (research / applied science / general), мест не публикует</t>
+        </is>
+      </c>
+      <c r="AI41" s="4" t="inlineStr">
         <is>
           <t>• Https://wu.edu.et
 • Https://wu.edu.et/wollo-universitys-president-signs-the-2018-e-c-key-performance-indicators-kpis-with-the-university-management-members/
 • Https://wu.edu.et/international-relation/ (empty page)
 • Https://www.wearetech.africa/en/fils-uk/news/tech/ethiopia-expands-space-program-with-2026-satellite-launch (general check: no Ethiopian university-built satellite)
-• Nanosats.csv (nation=Ethiopia: only ESSTI ET-SMART-RSS and cancelled AAiT ET-SAT)</t>
-        </is>
-      </c>
-      <c r="AI41" s="4" t="inlineStr">
+• Nanosats.csv (nation=Ethiopia: only ESSTI ET-SMART-RSS and cancelled AAiT ET-SAT)
+https://figshare.com/articles/preprint/Ranking_Web_of_Universities_webometrics_info_July_2026_edition/33062150</t>
+        </is>
+      </c>
+      <c r="AJ41" s="4" t="inlineStr">
         <is>
           <t>2026-10-05</t>
         </is>
       </c>
-      <c r="AJ41" s="4" t="inlineStr"/>
+      <c r="AK41" s="4" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AJ41"/>
+  <autoFilter ref="A1:AK41"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>